<commit_message>
Complete Grade 6 history teacher plans and update workbook
</commit_message>
<xml_diff>
--- a/standards/6th Grade/Grade_6_History_Curriculum_Standards.xlsx
+++ b/standards/6th Grade/Grade_6_History_Curriculum_Standards.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Course overview" sheetId="1" r:id="Rb6d205e096384aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 1" sheetId="2" r:id="R533219a8607a4d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 2" sheetId="3" r:id="R9427edbb19654bad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 3" sheetId="4" r:id="R98f19c2c455c4b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 4" sheetId="5" r:id="Rab2c91f367604a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Course overview" sheetId="1" r:id="Rf64fbe4d6e6a46d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 1" sheetId="2" r:id="Re4a90d1d55fd41d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 2" sheetId="3" r:id="R5774cae4b091439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 3" sheetId="4" r:id="R3ccae0edda084ab7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project 4" sheetId="5" r:id="Ra97bc7d472b441d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -359,7 +359,7 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="6" t="str">
-        <v>GRADE 6 HISTORY — Scope and sequence</v>
+        <v>GRADE 6 HISTORY — Scope, sequence and detailed lesson plans</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -404,7 +404,7 @@
         <v>Early humans, Mesopotamia, Egypt/Nubia, Israel, India, China, Greece and Rome.</v>
       </c>
       <c r="E5" s="11" t="str">
-        <v>Steps 1–4 scope and sequence drafted and reviewed. Detailed lesson plans (Step 5), student materials (Step 6) and classroom pacing remain to develop. One Tennessee chronology item remains unverified.</v>
+        <v>Steps 1–5 planning build: four projects and 32 detailed teacher lesson plans. Step 6 student packets, source-dependent checks and classroom pacing remain. Tennessee 6.39 chronology is Unverified; SSP.01 oral modality is Conditional.</v>
       </c>
     </row>
     <row r="6">
@@ -451,7 +451,7 @@
         <v>One evidence reconstruction board with a map/timeline, labeled artifacts, causal links and a revised explanation; each student supplies a private source-based argument.</v>
       </c>
       <c r="D9" s="11" t="str">
-        <v>Bounded source cards, maps and short adapted context readings; exact excerpts/access pending.</v>
+        <v>Bounded source selections and teacher plans; student adaptations and primary records remain to produce.</v>
       </c>
       <c r="E9" s="11" t="str">
         <v>Individual map/source reasoning and revised explanation; team quality reviewed separately.</v>
@@ -468,7 +468,7 @@
         <v>One shared atlas exhibit with three concise society panels and a common timeline/map. Every student completes evidence for all three; no specialist-only coverage.</v>
       </c>
       <c r="D10" s="13" t="str">
-        <v>Bounded source cards, maps and short adapted context readings; exact excerpts/access pending.</v>
+        <v>Bounded source selections and teacher plans; student adaptations and primary records remain to produce.</v>
       </c>
       <c r="E10" s="13" t="str">
         <v>Individual map/source reasoning and revised explanation; team quality reviewed separately.</v>
@@ -485,7 +485,7 @@
         <v>One paired China–Greece display with map/timeline, historical source panels, comparison table and investigation data; a short demonstration and individual explanation. Shadow data are supplied; the one practical investigation tests a water timer.</v>
       </c>
       <c r="D11" s="11" t="str">
-        <v>Bounded source cards, maps and short adapted context readings; exact excerpts/access pending.</v>
+        <v>Bounded source selections and teacher plans; student adaptations and primary records remain to produce.</v>
       </c>
       <c r="E11" s="11" t="str">
         <v>Individual map/source reasoning and revised explanation; team quality reviewed separately.</v>
@@ -502,7 +502,7 @@
         <v>One team council dossier with map/timeline, institutional comparison and causal evidence chart. Each student submits a short independent multi-cause account and fresh-source revision.</v>
       </c>
       <c r="D12" s="13" t="str">
-        <v>Bounded source cards, maps and short adapted context readings; exact excerpts/access pending.</v>
+        <v>Bounded source selections and teacher plans; student adaptations and primary records remain to produce.</v>
       </c>
       <c r="E12" s="13" t="str">
         <v>Individual map/source reasoning and revised explanation; team quality reviewed separately.</v>
@@ -552,7 +552,7 @@
         <v>Open the linked full course map for weekly progression, national routes, source records and Tennessee check.</v>
       </c>
       <c r="C17" s="11" t="str">
-        <v>Detailed lesson plans follow in Step 5.</v>
+        <v>All 32 detailed plans developed; Step 6 student packets and trials remain.</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -591,7 +591,7 @@
         <v>One paired historical display; one modern water-timer investigation, supplied shadow observations; historical and measured claims distinct.</v>
       </c>
       <c r="C20" s="13" t="str">
-        <v>Verify sources, procedure and accessible kits.</v>
+        <v>Procedure specified; pilot kits and complete source-dependent checks.</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -644,7 +644,7 @@
         <v>TN requirement / components</v>
       </c>
       <c r="B26" s="9" t="str">
-        <v>Outline and individual evidence destinations</v>
+        <v>Lesson and private evidence destinations</v>
       </c>
       <c r="C26" s="9" t="str">
         <v>Status</v>
@@ -666,7 +666,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D27" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E27" s="3"/>
     </row>
@@ -682,7 +682,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D28" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E28" s="3"/>
     </row>
@@ -698,7 +698,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D29" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E29" s="3"/>
     </row>
@@ -714,7 +714,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D30" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E30" s="3"/>
     </row>
@@ -730,7 +730,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D31" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E31" s="3"/>
     </row>
@@ -746,7 +746,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D32" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E32" s="3"/>
     </row>
@@ -762,7 +762,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D33" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E33" s="3"/>
     </row>
@@ -778,7 +778,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D34" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E34" s="3"/>
     </row>
@@ -794,11 +794,11 @@
         <v>Covered in plan</v>
       </c>
       <c r="D35" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E35" s="3"/>
     </row>
-    <row r="36" ht="74" customHeight="1">
+    <row r="36" ht="88" customHeight="1">
       <c r="A36" s="13" t="str">
         <v>6.10
 Describe the social hierarchy of ancient Mesopotamian society.</v>
@@ -810,7 +810,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D36" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E36" s="3"/>
     </row>
@@ -826,7 +826,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D37" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E37" s="3"/>
     </row>
@@ -842,7 +842,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D38" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E38" s="3"/>
     </row>
@@ -858,7 +858,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D39" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E39" s="3"/>
     </row>
@@ -874,7 +874,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D40" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E40" s="3"/>
     </row>
@@ -890,7 +890,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D41" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E41" s="3"/>
     </row>
@@ -906,7 +906,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D42" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E42" s="3"/>
     </row>
@@ -922,7 +922,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D43" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E43" s="3"/>
     </row>
@@ -938,7 +938,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D44" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E44" s="3"/>
     </row>
@@ -954,7 +954,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D45" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E45" s="3"/>
     </row>
@@ -970,7 +970,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D46" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E46" s="3"/>
     </row>
@@ -986,7 +986,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D47" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E47" s="3"/>
     </row>
@@ -1002,7 +1002,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D48" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E48" s="3"/>
     </row>
@@ -1018,7 +1018,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D49" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E49" s="3"/>
     </row>
@@ -1034,7 +1034,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D50" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E50" s="3"/>
     </row>
@@ -1050,7 +1050,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D51" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E51" s="3"/>
     </row>
@@ -1066,7 +1066,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D52" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E52" s="3"/>
     </row>
@@ -1082,7 +1082,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D53" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E53" s="3"/>
     </row>
@@ -1098,7 +1098,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D54" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E54" s="3"/>
     </row>
@@ -1114,7 +1114,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D55" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E55" s="3"/>
     </row>
@@ -1130,7 +1130,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D56" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E56" s="3"/>
     </row>
@@ -1146,7 +1146,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D57" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E57" s="3"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D58" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E58" s="3"/>
     </row>
@@ -1178,7 +1178,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D59" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E59" s="3"/>
     </row>
@@ -1194,7 +1194,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D60" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E60" s="3"/>
     </row>
@@ -1210,7 +1210,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D61" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E61" s="3"/>
     </row>
@@ -1226,7 +1226,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D62" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E62" s="3"/>
     </row>
@@ -1242,7 +1242,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D63" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E63" s="3"/>
     </row>
@@ -1258,7 +1258,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D64" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E64" s="3"/>
     </row>
@@ -1290,7 +1290,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D66" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E66" s="3"/>
     </row>
@@ -1306,7 +1306,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D67" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E67" s="3"/>
     </row>
@@ -1322,7 +1322,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D68" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E68" s="3"/>
     </row>
@@ -1338,7 +1338,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D69" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E69" s="3"/>
     </row>
@@ -1354,7 +1354,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D70" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E70" s="3"/>
     </row>
@@ -1370,7 +1370,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D71" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E71" s="3"/>
     </row>
@@ -1386,7 +1386,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D72" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E72" s="3"/>
     </row>
@@ -1402,7 +1402,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D73" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E73" s="3"/>
     </row>
@@ -1418,7 +1418,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D74" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E74" s="3"/>
     </row>
@@ -1434,7 +1434,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D75" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E75" s="3"/>
     </row>
@@ -1450,7 +1450,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D76" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E76" s="3"/>
     </row>
@@ -1466,7 +1466,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D77" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E77" s="3"/>
     </row>
@@ -1482,7 +1482,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D78" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E78" s="3"/>
     </row>
@@ -1498,7 +1498,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D79" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E79" s="3"/>
     </row>
@@ -1514,7 +1514,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D80" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E80" s="3"/>
     </row>
@@ -1530,7 +1530,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D81" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E81" s="3"/>
     </row>
@@ -1546,7 +1546,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D82" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E82" s="3"/>
     </row>
@@ -1562,7 +1562,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D83" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E83" s="3"/>
     </row>
@@ -1578,7 +1578,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D84" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E84" s="3"/>
     </row>
@@ -1594,7 +1594,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D85" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E85" s="3"/>
     </row>
@@ -1610,7 +1610,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D86" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E86" s="3"/>
     </row>
@@ -1626,7 +1626,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D87" s="11" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E87" s="3"/>
     </row>
@@ -1642,7 +1642,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D88" s="13" t="str">
-        <v>Verify the exact source packet and individual component checks in Step 5; produce and trial materials in Step 6.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E88" s="3"/>
     </row>
@@ -1655,10 +1655,10 @@
         <v>H1-W1-I, H1-W3-I, H2-W1-G, H3-W3-I, H4-W4-G</v>
       </c>
       <c r="C89" s="11" t="str">
-        <v>Covered in plan</v>
+        <v>Conditional</v>
       </c>
       <c r="D89" s="11" t="str">
-        <v>Recurring practice contributions; verify all source modalities and cumulative evidence in detailed planning. Oral-history study uses a sourced modern archaeology/discovery oral account, not a fabricated ancient eyewitness.</v>
+        <v>Written/artifact/map modalities specified. Select and verify the modern oral archaeology account before claiming the oral modality; written recollection alone is insufficient.</v>
       </c>
       <c r="E89" s="3"/>
     </row>
@@ -1674,7 +1674,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D90" s="13" t="str">
-        <v>Recurring practice contributions; verify all source modalities and cumulative evidence in detailed planning. Oral-history study uses a sourced modern archaeology/discovery oral account, not a fabricated ancient eyewitness.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E90" s="3"/>
     </row>
@@ -1690,7 +1690,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D91" s="11" t="str">
-        <v>Recurring practice contributions; verify all source modalities and cumulative evidence in detailed planning. Oral-history study uses a sourced modern archaeology/discovery oral account, not a fabricated ancient eyewitness.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E91" s="3"/>
     </row>
@@ -1706,7 +1706,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D92" s="13" t="str">
-        <v>Recurring practice contributions; verify all source modalities and cumulative evidence in detailed planning. Oral-history study uses a sourced modern archaeology/discovery oral account, not a fabricated ancient eyewitness.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E92" s="3"/>
     </row>
@@ -1722,7 +1722,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D93" s="11" t="str">
-        <v>Recurring practice contributions; verify all source modalities and cumulative evidence in detailed planning. Oral-history study uses a sourced modern archaeology/discovery oral account, not a fabricated ancient eyewitness.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E93" s="3"/>
     </row>
@@ -1738,7 +1738,7 @@
         <v>Covered in plan</v>
       </c>
       <c r="D94" s="13" t="str">
-        <v>Recurring practice contributions; verify all source modalities and cumulative evidence in detailed planning. Oral-history study uses a sourced modern archaeology/discovery oral account, not a fabricated ancient eyewitness.</v>
+        <v>Detailed teaching and private assessment specification exists at named routes. Produce/check source packets and response keys, then observe individual components; route coverage is not demonstrated mastery.</v>
       </c>
       <c r="E94" s="3"/>
     </row>
@@ -1776,12 +1776,12 @@
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" ht="74" customHeight="1">
+    <row r="99" ht="88" customHeight="1">
       <c r="A99" s="11" t="str">
-        <v>Historical depth and calendar</v>
+        <v>Material production</v>
       </c>
       <c r="B99" s="11" t="str">
-        <v>16 weeks gives a survey across seven major society contexts. Confirm expected depth and actual dates; trial H2-W3 and H3-W2 before detailed expansion. Additional depth may need more time.</v>
+        <v>Step 6: produce the 32 bounded source packets, accessible maps/cards, models, developing responses, held-back cases and response keys from the detailed specifications. Check primary-object provenance and exact excerpt fit.</v>
       </c>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
@@ -1789,10 +1789,10 @@
     </row>
     <row r="100" ht="74" customHeight="1">
       <c r="A100" s="13" t="str">
-        <v>Exact source packets</v>
+        <v>Historical chronology</v>
       </c>
       <c r="B100" s="13" t="str">
-        <v>Step 5 selects creator/date/place/purpose/audience, excerpt boundaries and contrasting viewpoints; Step 6 builds accessible texts/images, fresh cases and answer/scoring guidance.</v>
+        <v>TN 6.39 remains Unverified: date documented Han achievements and later printing separately; verify compass/porcelain attribution before certifying these components.</v>
       </c>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
@@ -1800,10 +1800,10 @@
     </row>
     <row r="101" ht="74" customHeight="1">
       <c r="A101" s="11" t="str">
-        <v>H3 historical chronology</v>
+        <v>Oral modality</v>
       </c>
       <c r="B101" s="11" t="str">
-        <v>TN 6.39 groups printing with Han achievements. Teach evidence-based dates; keep the disputed attribution Unverified pending interpretation. Verify all invention chronology.</v>
+        <v>SSP.01 is Conditional until a real 60–90-second modern archaeology oral account has verified speaker/date/context and transcript. A written discovery record does not satisfy oral evidence.</v>
       </c>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
@@ -1811,10 +1811,10 @@
     </row>
     <row r="102" ht="74" customHeight="1">
       <c r="A102" s="13" t="str">
-        <v>H3 investigation access</v>
+        <v>Investigation</v>
       </c>
       <c r="B102" s="13" t="str">
-        <v>Verify Greek clock source access; choose exact Han primary record. Prepare adult-made water-timer kits, equivalent participation and supplied shadow data with provenance.</v>
+        <v>Pilot six adult-prepared water timers and labeled supplied shadow data; choose the Han primary artifact record. MacTutor provides the selected Greek scholarly context.</v>
       </c>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
@@ -1822,10 +1822,10 @@
     </row>
     <row r="103" ht="74" customHeight="1">
       <c r="A103" s="11" t="str">
-        <v>Religion and historical interpretation</v>
+        <v>Pacing and enrollment</v>
       </c>
       <c r="B103" s="11" t="str">
-        <v>Use matched academic religion profiles, accurate sacred-text attribution and scholarly context; keep tradition, belief and corroborated historical evidence distinct.</v>
+        <v>All 32 budgets total 90 minutes with at least 30 minutes project work. Assume 24 students/six groups; trial H2-W3 and H3-W2 with actual readers. Keep no required homework.</v>
       </c>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
@@ -1833,22 +1833,18 @@
     </row>
     <row r="104" ht="60" customHeight="1">
       <c r="A104" s="13" t="str">
-        <v>Enrollment and observation</v>
+        <v>Program boundary</v>
       </c>
       <c r="B104" s="13" t="str">
-        <v>Assume 24 learners/six teams. Confirm class size and observation capacity before detailed clocks. No required homework.</v>
+        <v>Selected NCSS themes/C3 contributions only; schoolwide grade-band ownership, accreditor identity and criteria remain separate.</v>
       </c>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
     </row>
-    <row r="105" ht="88" customHeight="1">
-      <c r="A105" s="11" t="str">
-        <v>Program boundary</v>
-      </c>
-      <c r="B105" s="11" t="str">
-        <v>Selected NCSS themes/C3 contributions support this ancient-history term. Other geography/economics, contemporary civics and complete Grades 6–8 expectations require schoolwide ownership. Accreditor identity/criteria remain to supply separately.</v>
-      </c>
+    <row r="105">
+      <c r="A105" s="3"/>
+      <c r="B105" s="3"/>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
@@ -1860,80 +1856,80 @@
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
     </row>
-    <row r="107">
-      <c r="A107" s="3"/>
-      <c r="B107" s="3"/>
-      <c r="C107" s="3"/>
-      <c r="D107" s="3"/>
-      <c r="E107" s="3"/>
-    </row>
-    <row r="108" ht="30" customHeight="1">
-      <c r="A108" s="6" t="str">
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="6" t="str">
         <v>Official framework and compliance sources</v>
       </c>
-      <c r="B108" s="6"/>
-      <c r="C108" s="6"/>
-      <c r="D108" s="6"/>
-      <c r="E108" s="6"/>
-    </row>
-    <row r="109" ht="55" customHeight="1">
-      <c r="A109" s="9" t="str">
+      <c r="B107" s="6"/>
+      <c r="C107" s="6"/>
+      <c r="D107" s="6"/>
+      <c r="E107" s="6"/>
+    </row>
+    <row r="108" ht="55" customHeight="1">
+      <c r="A108" s="9" t="str">
         <v>Source</v>
       </c>
-      <c r="B109" s="9" t="str">
+      <c r="B108" s="9" t="str">
         <v>Full title</v>
       </c>
-      <c r="C109" s="9" t="str">
+      <c r="C108" s="9" t="str">
         <v>Assigned use</v>
       </c>
-      <c r="D109" s="9" t="str">
+      <c r="D108" s="9" t="str">
         <v>Access / limits</v>
       </c>
+      <c r="E108" s="3"/>
+    </row>
+    <row r="109" ht="74" customHeight="1">
+      <c r="A109" s="11" t="str">
+        <v>NCSS</v>
+      </c>
+      <c r="B109" s="14" t="str">
+        <v>NCSS National Curriculum Standards for Social Studies (2010): public executive summary and themes</v>
+      </c>
+      <c r="C109" s="11" t="str">
+        <v>Ten-theme organizing framework; public middle-grades discussion. Full proprietary middle-grades performance expectations are not reproduced or individually certified.</v>
+      </c>
+      <c r="D109" s="11" t="str">
+        <v>Official public framework reviewed 2026-10-03.</v>
+      </c>
       <c r="E109" s="3"/>
     </row>
-    <row r="110" ht="74" customHeight="1">
-      <c r="A110" s="11" t="str">
-        <v>NCSS</v>
-      </c>
-      <c r="B110" s="14" t="str">
-        <v>NCSS National Curriculum Standards for Social Studies (2010): public executive summary and themes</v>
-      </c>
-      <c r="C110" s="11" t="str">
-        <v>Ten-theme organizing framework; public middle-grades discussion. Full proprietary middle-grades performance expectations are not reproduced or individually certified.</v>
-      </c>
-      <c r="D110" s="11" t="str">
-        <v>Official public framework reviewed 2026-10-03.</v>
+    <row r="110" ht="60" customHeight="1">
+      <c r="A110" s="13" t="str">
+        <v>C3</v>
+      </c>
+      <c r="B110" s="15" t="str">
+        <v>NCSS C3 Framework (2013), Grades 6–8 inquiry indicators</v>
+      </c>
+      <c r="C110" s="13" t="str">
+        <v>Questions, maps, institutions, historical context/perspective/evidence/causation, source evaluation and communication. Selected indicators only.</v>
+      </c>
+      <c r="D110" s="13" t="str">
+        <v>Official PDF reviewed online 2026-10-03; selected grade-band contributions, not a complete C3 band claim.</v>
       </c>
       <c r="E110" s="3"/>
     </row>
-    <row r="111" ht="60" customHeight="1">
-      <c r="A111" s="13" t="str">
-        <v>C3</v>
-      </c>
-      <c r="B111" s="15" t="str">
-        <v>NCSS C3 Framework (2013), Grades 6–8 inquiry indicators</v>
-      </c>
-      <c r="C111" s="13" t="str">
-        <v>Questions, maps, institutions, historical context/perspective/evidence/causation, source evaluation and communication. Selected indicators only.</v>
-      </c>
-      <c r="D111" s="13" t="str">
-        <v>Official PDF reviewed online 2026-10-03; selected grade-band contributions, not a complete C3 band claim.</v>
+    <row r="111" ht="55" customHeight="1">
+      <c r="A111" s="11" t="str">
+        <v>TN</v>
+      </c>
+      <c r="B111" s="14" t="str">
+        <v>Tennessee Social Studies Standards: implementation 2027–28</v>
+      </c>
+      <c r="C111" s="11" t="str">
+        <v>Local official PDF pages 81–98: SSP.01–06 and content 6.01–6.62.</v>
+      </c>
+      <c r="D111" s="11" t="str">
+        <v>2024 adoption, 2027–28 implementation. Separate content check; 6.39 chronology unresolved.</v>
       </c>
       <c r="E111" s="3"/>
     </row>
-    <row r="112" ht="55" customHeight="1">
-      <c r="A112" s="11" t="str">
-        <v>TN</v>
-      </c>
-      <c r="B112" s="14" t="str">
-        <v>Tennessee Social Studies Standards: implementation 2027–28</v>
-      </c>
-      <c r="C112" s="11" t="str">
-        <v>Local official PDF pages 81–98: SSP.01–06 and content 6.01–6.62.</v>
-      </c>
-      <c r="D112" s="11" t="str">
-        <v>2024 adoption, 2027–28 implementation. Separate content check; 6.39 chronology unresolved.</v>
-      </c>
+    <row r="112">
+      <c r="A112" s="3"/>
+      <c r="B112" s="3"/>
+      <c r="C112" s="3"/>
+      <c r="D112" s="3"/>
       <c r="E112" s="3"/>
     </row>
     <row r="113">
@@ -2069,7 +2065,7 @@
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A97:E97"/>
-    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A107:E107"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A9" location="'Project 1'!A2"/>
@@ -2077,9 +2073,9 @@
     <hyperlink ref="A11" location="'Project 3'!A2"/>
     <hyperlink ref="A12" location="'Project 4'!A2"/>
     <hyperlink ref="B17" r:id="historyLink4"/>
-    <hyperlink ref="B110" r:id="historyLink5"/>
-    <hyperlink ref="B111" r:id="historyLink6"/>
-    <hyperlink ref="B112" r:id="historyLink7"/>
+    <hyperlink ref="B109" r:id="historyLink5"/>
+    <hyperlink ref="B110" r:id="historyLink6"/>
+    <hyperlink ref="B111" r:id="historyLink7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2137,11 +2133,11 @@
     </row>
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="3" t="str">
-        <v>Step 4 block outlines</v>
+        <v>Step 5 teacher plans</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="str">
-        <v>Detailed procedures, exact source excerpts, examples and assessment prompts remain Step 5 work.</v>
+        <v>Full procedures, worked examples, private prompts and clocks in linked plans; Step 6 packets and trials remain.</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2190,7 +2186,7 @@
         <v>Standards - national</v>
       </c>
     </row>
-    <row r="7" ht="158" customHeight="1">
+    <row r="7" ht="200" customHeight="1">
       <c r="A7" s="16" t="str">
         <v>H1-W1-I
 Week 1 | Individual</v>
@@ -2201,26 +2197,27 @@
       </c>
       <c r="C7" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 3.1 Early Civilizations: evidence/timeline introduction, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D7" s="11" t="str">
-        <v>Contrast an artifact with a modern caption; place three dated examples on a timeline and distinguish observation from inference.</v>
+        <v>Contrast an artifact with a modern caption; place three dated examples on a timeline and distinguish observation from inference. Example: On different dates, 3000 BCE precedes 1000 BCE; circa signals approximation. An object is primary evidence for its manufacture, while a present caption is secondary interpretation; neither alone establishes every user's beliefs.</v>
       </c>
       <c r="E7" s="11" t="str">
-        <v>Annotate a timeline; classify sources; pose the settlement inquiry and choose two sources that could answer a supporting question.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate a timeline; classify sources; pose the settlement inquiry and choose two sources that could answer a supporting question. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F7" s="11" t="str">
         <v>Collect: Individual dated sequence, source classification and justified source choice.
-Judge: Correct chronology and labels; source choice matches question; inference exceeds neither object nor caption.
-Feedback/support: If oldest BCE is reversed, model an ordered number line and recheck new dates; offer a labeled chronology strip.</v>
+Prompt: Order 2400 BCE, 1800 BCE and 500 CE. Explain circa. Classify an excavated tablet and a modern museum caption. Which two source types could answer how a settlement obtained food, and how would they offer different perspectives?
+Criteria: Correct chronology and labels; source choice matches question; inference exceeds neither object nor caption.
+Response to difficulty: If oldest BCE is reversed, model an ordered number line and recheck new dates; offer a labeled chronology strip.</v>
       </c>
       <c r="G7" s="11" t="str">
-        <v>Prepare timeline cards and provenance labels; save the inquiry/source log for all projects.</v>
+        <v>Prepare timeline cards and provenance labels; save the inquiry/source log for all projects. Carry saved private evidence and unresolved component notes to H1-W1-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H7" s="11" t="str">
-        <v>Teach / revisit: BCE/CE, BC/AD, circa, decades/centuries; primary/secondary sources and archaeological inference.
-Practice: Annotate a timeline; classify sources; pose the settlement inquiry and choose two sources that could answer a supporting question.
+        <v>Teach / revisit: Read time and question the evidence
+Practice: source/context reasoning through the project task.
 Check: Individual dated sequence, source classification and justified source choice.
 Builds on: Grade 5 maps, sequence and evidence language.</v>
       </c>
@@ -2228,10 +2225,10 @@
         <v>C3 Primary: D2.His.1.6-8, D2.His.9.6-8, D1.5.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="8" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="8" ht="214" customHeight="1">
       <c r="A8" s="17" t="str">
         <v>H1-W1-G
 Week 1 | Group</v>
@@ -2242,26 +2239,27 @@
       </c>
       <c r="C8" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 2.3 The Neolithic Revolution: Development of Agriculture and How Farming Changed Human Experience, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D8" s="13" t="str">
-        <v>Model a multi-cause chain on a different settlement; explain that mobile lifeways did not simply disappear everywhere.</v>
+        <v>Model a multi-cause chain on a different settlement; explain that mobile lifeways did not simply disappear everywhere. Example: A hypothetical settlement has grain storage and weaving tools: storage may support specialized work, but flood damage could interrupt it. Tools remain in both cases; settlement does not imply all mobile communities vanished.</v>
       </c>
       <c r="E8" s="13" t="str">
-        <v>Compare two evidence sets; construct a settlement-change chain; teams propose and challenge two explanations.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Compare two evidence sets; construct a settlement-change chain; teams propose and challenge two explanations. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F8" s="13" t="str">
         <v>Collect: Private continuity/change comparison and one evidence-supported cause/effect chain.
-Judge: Distinguishes material evidence from assumptions; includes both continuity and change without ranking people.
-Feedback/support: If surplus is automatic, add a failed-harvest case and revise; use pictured process cards with a fresh explanation.</v>
+Prompt: Use both site cases to explain one continuity and two changes between mobile and settled lives. Connect domestication, surplus and specialization; explain why a failed harvest weakens an automatic-surplus claim.
+Criteria: Distinguishes material evidence from assumptions; includes both continuity and change without ranking people.
+Response to difficulty: If surplus is automatic, add a failed-harvest case and revise; use pictured process cards with a fresh explanation.</v>
       </c>
       <c r="G8" s="13" t="str">
-        <v>Create bounded site cases and preserve individual chains on the reconstruction board.</v>
+        <v>Create bounded site cases and preserve individual chains on the reconstruction board. Carry saved private evidence and unresolved component notes to H1-W2-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H8" s="13" t="str">
-        <v>Teach / revisit: Paleolithic tools, fire, hunting, shelter and mobility; Neolithic agriculture, domestication, surplus, barter, clothing/shelter and specialized work.
-Practice: Compare two evidence sets; construct a settlement-change chain; teams propose and challenge two explanations.
+        <v>Teach / revisit: Compare mobile and settled lives
+Practice: source/context reasoning through the project task.
 Check: Private continuity/change comparison and one evidence-supported cause/effect chain.
 Builds on: H1-W1-I source and chronology routines.</v>
       </c>
@@ -2269,10 +2267,10 @@
         <v>C3 Primary: D2.His.2.6-8, D2.His.14.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T7, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="9" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="9" ht="200" customHeight="1">
       <c r="A9" s="16" t="str">
         <v>H1-W2-I
 Week 2 | Individual</v>
@@ -2283,26 +2281,27 @@
       </c>
       <c r="C9" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 3.2 Ancient Mesopotamia: geography and settlement, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D9" s="11" t="str">
-        <v>Model map selection by purpose/date; explain how irrigation modifies the environment rather than saying rivers guarantee prosperity.</v>
+        <v>Model map selection by purpose/date; explain how irrigation modifies the environment rather than saying rivers guarantee prosperity. Example: A hypothetical riverbank provides water but exposes fields to floods; a canal is a human adaptation with labor and maintenance costs. A map's date and purpose limit boundary claims.</v>
       </c>
       <c r="E9" s="11" t="str">
-        <v>Label a bounded regional map; compare two possible settlement locations; annotate benefits, risks and human adaptations.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Label a bounded regional map; compare two possible settlement locations; annotate benefits, risks and human adaptations. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F9" s="11" t="str">
         <v>Collect: Individual map and location explanation using two features and an adaptation.
-Judge: Features are positioned meaningfully; cultural/economic decisions and environmental effects are connected.
-Feedback/support: If modern borders become ancient boundaries, compare dated maps then recheck; provide readable relief and text equivalents.</v>
+Prompt: Label Tigris, Euphrates, Zagros, Mediterranean and Persian Gulf. Recommend one of the two proposed settlement locations using two mapped features, a risk and an adaptation that changes the environment.
+Criteria: Features are positioned meaningfully; cultural/economic decisions and environmental effects are connected.
+Response to difficulty: If modern borders become ancient boundaries, compare dated maps then recheck; provide readable relief and text equivalents.</v>
       </c>
       <c r="G9" s="11" t="str">
-        <v>Prepare relief/water maps and carry location decisions into the city model.</v>
+        <v>Prepare relief/water maps and carry location decisions into the city model. Carry saved private evidence and unresolved component notes to H1-W2-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H9" s="11" t="str">
-        <v>Teach / revisit: Tigris, Euphrates, Zagros, Mediterranean and Persian Gulf; rainfall/floods, water access, irrigation and agricultural risk.
-Practice: Label a bounded regional map; compare two possible settlement locations; annotate benefits, risks and human adaptations.
+        <v>Teach / revisit: Locate the Fertile Crescent
+Practice: source/context reasoning through the project task.
 Check: Individual map and location explanation using two features and an adaptation.
 Builds on: Timeline and cause/effect reasoning.</v>
       </c>
@@ -2310,10 +2309,10 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.Geo.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T3 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="10" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="10" ht="214" customHeight="1">
       <c r="A10" s="17" t="str">
         <v>H1-W2-G
 Week 2 | Group</v>
@@ -2324,26 +2323,27 @@
       </c>
       <c r="C10" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 3.2 Ancient Mesopotamia: agriculture, city-states and technologies, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D10" s="13" t="str">
-        <v>Model surplus-to-specialization with alternatives; show institutions allocating water/work without a modern market assumption.</v>
+        <v>Model surplus-to-specialization with alternatives; show institutions allocating water/work without a modern market assumption. Example: A teacher-created canal diagram links organized maintenance to water delivery, yield and exchanged surplus. A broken channel interrupts the mechanism; drawing a wheel without explaining transport provides no causal evidence.</v>
       </c>
       <c r="E10" s="13" t="str">
-        <v>Build a city systems diagram; match each civilization characteristic to evidence; analyze agricultural tools and a trade route.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Build a city systems diagram; match each civilization characteristic to evidence; analyze agricultural tools and a trade route. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F10" s="13" t="str">
         <v>Collect: Each student explains an institution and two links among agriculture, labor and exchange.
-Judge: All seven characteristics appear with evidence; mechanisms explain tool and trade effects; no single-cause story.
-Feedback/support: If diagram is only pictures, add labeled causal verbs and recheck a new link; offer a systems organizer.</v>
+Prompt: Annotate all seven civilization characteristics on your city diagram. Explain how irrigation and one transport technology affect specialization and trade; identify the institution organizing work and a possible disruption.
+Criteria: All seven characteristics appear with evidence; mechanisms explain tool and trade effects; no single-cause story.
+Response to difficulty: If diagram is only pictures, add labeled causal verbs and recheck a new link; offer a systems organizer.</v>
       </c>
       <c r="G10" s="13" t="str">
-        <v>Prepare verified agriculture/technology cards; keep the same city board for law and belief sources.</v>
+        <v>Prepare verified agriculture/technology cards; keep the same city board for law and belief sources. Carry saved private evidence and unresolved component notes to H1-W3-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H10" s="13" t="str">
-        <v>Teach / revisit: Food supply, technology, culture, writing, religion, government and social structure; irrigation/metallurgy/animals/wheel/sail/plow; surplus, trade, transport and city-states.
-Practice: Build a city systems diagram; match each civilization characteristic to evidence; analyze agricultural tools and a trade route.
+        <v>Teach / revisit: Explain how an early city worked
+Practice: source/context reasoning through the project task.
 Check: Each student explains an institution and two links among agriculture, labor and exchange.
 Builds on: Map, adaptation and settlement chains.</v>
       </c>
@@ -2351,10 +2351,10 @@
         <v>C3 Primary: D2.His.14.6-8, D2.Civ.6.6-8
 Supporting: D3.1.6-8
 NCSS themes: T5, T7, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="11" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="11" ht="214" customHeight="1">
       <c r="A11" s="16" t="str">
         <v>H1-W3-I
 Week 3 | Individual</v>
@@ -2365,26 +2365,27 @@
       </c>
       <c r="C11" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 3.2 Ancient Mesopotamia: institutions, religion and writing, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D11" s="11" t="str">
-        <v>Compare a ruler inscription with an archaeological account; teach how elite sources preserve some voices and omit others.</v>
+        <v>Compare a ruler inscription with an archaeological account; teach how elite sources preserve some voices and omit others. Example: A hypothetical royal inscription praises a ruler: its audience/purpose may explain emphasis on victories. A worker's experience remains unknown; an epic can reveal ideals without proving every narrated event.</v>
       </c>
       <c r="E11" s="11" t="str">
-        <v>Annotate a social-role/source chart; distinguish belief from historical claim; connect cuneiform and architecture to institutions.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate a social-role/source chart; distinguish belief from historical claim; connect cuneiform and architecture to institutions. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F11" s="11" t="str">
         <v>Collect: Individual explanation of power/social position and one source-perspective limitation.
-Judge: Defines government forms; explains daily-life effects and belief context; treats an epic as literature/evidence rather than a literal event log.
-Feedback/support: If a ruler speaks for everyone, identify absent groups and recheck a different source; use role/source labels.</v>
+Prompt: Compare city-state, monarchy and empire. Explain how social position affects daily life; use a tablet, ziggurat or epic to connect belief and institution. Whose perspective is preserved and whose is missing?
+Criteria: Defines government forms; explains daily-life effects and belief context; treats an epic as literature/evidence rather than a literal event log.
+Response to difficulty: If a ruler speaks for everyone, identify absent groups and recheck a different source; use role/source labels.</v>
       </c>
       <c r="G11" s="11" t="str">
-        <v>Select translations and exact object records; distinguish first-known empire claims and Gilgamesh traditions from universal absolutes.</v>
+        <v>Select translations and exact object records; distinguish first-known empire claims and Gilgamesh traditions from universal absolutes. Carry saved private evidence and unresolved component notes to H1-W3-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H11" s="11" t="str">
-        <v>Teach / revisit: City-state versus monarchy/empire; Mesopotamian social hierarchy; polytheism and nature; writing, tablets, ziggurats and Gilgamesh.
-Practice: Annotate a social-role/source chart; distinguish belief from historical claim; connect cuneiform and architecture to institutions.
+        <v>Teach / revisit: Read authority, hierarchy and beliefs
+Practice: source/context reasoning through the project task.
 Check: Individual explanation of power/social position and one source-perspective limitation.
 Builds on: Institutions and artifact inference.</v>
       </c>
@@ -2392,10 +2393,10 @@
         <v>C3 Primary: D2.Civ.6.6-8, D2.His.4.6-8, D2.His.6.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T4, T5, T6 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="12" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="12" ht="242" customHeight="1">
       <c r="A12" s="17" t="str">
         <v>H1-W3-G
 Week 3 | Group</v>
@@ -2405,27 +2406,28 @@
 Hammurabi, written law, status-dependent justice; corroboration and source purpose.</v>
       </c>
       <c r="C12" s="15" t="str">
-        <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+        <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource; Fordham Ancient History Sourcebook — Code of Hammurabi, L. W. King translation
+In class: 150–250 words of attributed teacher adaptation from 3.2 Ancient Mesopotamia: Hammurabi; paired numbered laws 8 and 48 in Fordham translation, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D12" s="13" t="str">
-        <v>Model inferring audience/purpose by comparing a law excerpt with a second account; written law does not prove equal enforcement.</v>
+        <v>Model inferring audience/purpose by comparing a law excerpt with a second account; written law does not prove equal enforcement. Example: Law 48 addresses harvest failure and debt obligations. A written rule supports a claim about prescribed responses, while enforcement needs other evidence. Compare a different rule before inferring equal treatment.</v>
       </c>
       <c r="E12" s="13" t="str">
-        <v>Compare two adapted laws and contextual evidence; explain affected groups; revise an unsupported equality claim.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Compare two adapted laws and contextual evidence; explain affected groups; revise an unsupported equality claim. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F12" s="13" t="str">
         <v>Collect: Private corroborated source-purpose inference and a claim with one limitation.
-Judge: Cites both sources; explains relevance and status differences; avoids reading modern equality into the text.
-Feedback/support: If paraphrase becomes endorsement, separate description from evaluation and recheck; offer side-by-side source chunks.</v>
+Prompt: Compare Hammurabi laws 8 and 48 with the artifact/context account. What purpose and audience can you infer? Explain why written rules do not prove equal treatment or actual enforcement.
+Criteria: Cites both sources; explains relevance and status differences; avoids reading modern equality into the text.
+Response to difficulty: If paraphrase becomes endorsement, separate description from evaluation and recheck; offer side-by-side source chunks.</v>
       </c>
       <c r="G12" s="13" t="str">
-        <v>Prepare verified translator/date/section labels and carry law evidence into reconstruction.</v>
+        <v>Prepare verified translator/date/section labels and carry law evidence into reconstruction. Carry saved private evidence and unresolved component notes to H1-W4-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H12" s="13" t="str">
-        <v>Teach / revisit: Hammurabi, written law, status-dependent justice; corroboration and source purpose.
-Practice: Compare two adapted laws and contextual evidence; explain affected groups; revise an unsupported equality claim.
+        <v>Teach / revisit: Compare law and lived experience
+Practice: source/context reasoning through the project task.
 Check: Private corroborated source-purpose inference and a claim with one limitation.
 Builds on: Hierarchy and source perspective.</v>
       </c>
@@ -2433,10 +2435,10 @@
         <v>C3 Primary: D2.His.11.6-8, D3.2.6-8, D3.3.6-8
 Supporting: D3.1.6-8
 NCSS themes: T6, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="13" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="13" ht="200" customHeight="1">
       <c r="A13" s="16" t="str">
         <v>H1-W4-I
 Week 4 | Individual</v>
@@ -2447,26 +2449,27 @@
       </c>
       <c r="C13" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from Reuse H1 source log; no new long reading, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D13" s="11" t="str">
-        <v>Model a supported claim with an alternative explanation and an evidence limit on a different site.</v>
+        <v>Model a supported claim with an alternative explanation and an evidence limit on a different site. Example: Use a different settlement case: map access plus storage evidence support an exchange explanation, but stored goods alone do not identify ownership. A competing seasonal-storage interpretation narrows the conclusion.</v>
       </c>
       <c r="E13" s="11" t="str">
-        <v>Finish existing board annotations; independently argue which explanation fits; use peer credibility feedback to revise.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Finish existing board annotations; independently argue which explanation fits; use peer credibility feedback to revise. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F13" s="11" t="str">
         <v>Collect: Individual argument from at least two source types plus one substantive revision.
-Judge: Evidence supports mechanisms and chronology; alternative is fairly considered; uncertainty remains visible.
-Feedback/support: If claim repeats a caption, ask how evidence supports it; recheck an unfamiliar artifact; allow oral reasoning with citations.</v>
+Prompt: Write a 150–250-word or equivalent reconstruction argument using a map and artifact/text. Explain two interacting causes of city development, consider an alternative and identify a source limitation. Revise one causal link after feedback.
+Criteria: Evidence supports mechanisms and chronology; alternative is fairly considered; uncertainty remains visible.
+Response to difficulty: If claim repeats a caption, ask how evidence supports it; recheck an unfamiliar artifact; allow oral reasoning with citations.</v>
       </c>
       <c r="G13" s="11" t="str">
-        <v>Prepare short fresh artifact check and archive each student’s source choices.</v>
+        <v>Prepare short fresh artifact check and archive each student’s source choices. Carry saved private evidence and unresolved component notes to H1-W4-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H13" s="11" t="str">
-        <v>Teach / revisit: Synthesize chronology, geography, technology, institutions and competing settlement explanations.
-Practice: Finish existing board annotations; independently argue which explanation fits; use peer credibility feedback to revise.
+        <v>Teach / revisit: Defend the city reconstruction
+Practice: source/context reasoning through the project task.
 Check: Individual argument from at least two source types plus one substantive revision.
 Builds on: All H1 source and city-system work.</v>
       </c>
@@ -2474,10 +2477,10 @@
         <v>C3 Primary: D2.His.16.6-8, D4.1.6-8, D4.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T3, T5 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="14" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="14" ht="200" customHeight="1">
       <c r="A14" s="17" t="str">
         <v>H1-W4-G
 Week 4 | Group</v>
@@ -2488,26 +2491,27 @@
       </c>
       <c r="C14" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Art of the Ancient Near East: educator resource
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from Held-back artifact/caption; reuse H1 source log, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D14" s="13" t="str">
-        <v>Demonstrate critiquing sequence and causal links without judging decorative design.</v>
+        <v>Demonstrate critiquing sequence and causal links without judging decorative design. Example: A held-back tool's worn edge supports use but not the user's social rank. Add a dated caption before drawing a broader city-life inference.</v>
       </c>
       <c r="E14" s="13" t="str">
-        <v>Teams give concise reconstruction walkthroughs; each learner responds to a new artifact/caption; revise one causal link.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Teams give concise reconstruction walkthroughs; each learner responds to a new artifact/caption; revise one causal link. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F14" s="13" t="str">
         <v>Collect: Private new-source inference, limitation and teacher-recorded explanation; team board reviewed separately.
-Judge: New evidence is contextualized; explanation order is coherent; revision changes reasoning.
-Feedback/support: If new object is dated incorrectly, use timeline/source clinic and a second card; carry missing evidence forward.</v>
+Prompt: Using the held-back artifact/caption, record an observation, a contextual inference and a limit. Explain whether it strengthens or weakens a link on your city board; justify the change independently.
+Criteria: New evidence is contextualized; explanation order is coherent; revision changes reasoning.
+Response to difficulty: If new object is dated incorrectly, use timeline/source clinic and a second card; carry missing evidence forward.</v>
       </c>
       <c r="G14" s="13" t="str">
-        <v>Save map/source log and individual unresolved needs for H2; prepare source packets before detailed lessons.</v>
+        <v>Save map/source log and individual unresolved needs for H2; prepare source packets before detailed lessons. Carry saved private evidence and unresolved component notes to H2-W1-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H14" s="13" t="str">
-        <v>Teach / revisit: Evidence conference, new artifact interpretation and unresolved inquiry.
-Practice: Teams give concise reconstruction walkthroughs; each learner responds to a new artifact/caption; revise one causal link.
+        <v>Teach / revisit: Review competing reconstructions
+Practice: source/context reasoning through the project task.
 Check: Private new-source inference, limitation and teacher-recorded explanation; team board reviewed separately.
 Builds on: Source credibility, causal argument and timeline.</v>
       </c>
@@ -2515,7 +2519,7 @@
         <v>C3 Primary: D4.2.6-8, D4.5.6-8, D2.His.10.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
       </c>
     </row>
     <row r="15">
@@ -2572,7 +2576,7 @@
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
     </row>
-    <row r="19" ht="102" customHeight="1">
+    <row r="19" ht="116" customHeight="1">
       <c r="A19" s="11" t="str">
         <v>H1-W1-I</v>
       </c>
@@ -2584,7 +2588,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D19" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -2592,7 +2596,7 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" ht="102" customHeight="1">
+    <row r="20" ht="116" customHeight="1">
       <c r="A20" s="13" t="str">
         <v>H1-W1-G</v>
       </c>
@@ -2604,7 +2608,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D20" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -2612,7 +2616,7 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" ht="102" customHeight="1">
+    <row r="21" ht="116" customHeight="1">
       <c r="A21" s="11" t="str">
         <v>H1-W2-I</v>
       </c>
@@ -2624,7 +2628,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D21" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -2632,7 +2636,7 @@
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" ht="102" customHeight="1">
+    <row r="22" ht="116" customHeight="1">
       <c r="A22" s="13" t="str">
         <v>H1-W2-G</v>
       </c>
@@ -2644,7 +2648,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D22" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -2652,7 +2656,7 @@
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" ht="102" customHeight="1">
+    <row r="23" ht="116" customHeight="1">
       <c r="A23" s="11" t="str">
         <v>H1-W3-I</v>
       </c>
@@ -2664,7 +2668,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D23" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -2672,7 +2676,7 @@
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
     </row>
-    <row r="24" ht="102" customHeight="1">
+    <row r="24" ht="116" customHeight="1">
       <c r="A24" s="13" t="str">
         <v>H1-W3-G</v>
       </c>
@@ -2684,7 +2688,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D24" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -2692,7 +2696,7 @@
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
     </row>
-    <row r="25" ht="102" customHeight="1">
+    <row r="25" ht="116" customHeight="1">
       <c r="A25" s="11" t="str">
         <v>H1-W4-I</v>
       </c>
@@ -2704,7 +2708,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D25" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -2712,7 +2716,7 @@
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
     </row>
-    <row r="26" ht="102" customHeight="1">
+    <row r="26" ht="116" customHeight="1">
       <c r="A26" s="13" t="str">
         <v>H1-W4-G</v>
       </c>
@@ -2724,7 +2728,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D26" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -2788,7 +2792,7 @@
     </row>
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="11" t="str">
-        <v>Project outline</v>
+        <v>Detailed project plan</v>
       </c>
       <c r="B31" s="14" t="str">
         <v>H1 First Cities Evidence Dig</v>
@@ -2797,7 +2801,7 @@
         <v>One evidence reconstruction board with a map/timeline, labeled artifacts, causal links and a revised explanation; each student supplies a private source-based argument.</v>
       </c>
       <c r="D31" s="11" t="str">
-        <v>Step 4 outline exists; detailed Step 5 lessons pending.</v>
+        <v>Eight detailed Step 5 plans developed; Step 6 materials remain.</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -2816,7 +2820,7 @@
         <v>Teacher background: early humans, river-valley societies, ancient Israel/India/China/Greece/Rome. Select topic sections and primary-source boxes; prepare short attributed student adaptations.</v>
       </c>
       <c r="D32" s="13" t="str">
-        <v>Teacher reference located; exact excerpts, dates, image rights, reading fit and source packets remain Step 5/6 work. Do not assign whole college chapters.</v>
+        <v>Named section selections specified in all 32 detailed plans. Bounded Grade 6 adaptations and source boxes remain Step 6; do not assign whole college chapters.</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -2843,11 +2847,19 @@
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
     </row>
-    <row r="34">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
+    <row r="34" ht="88" customHeight="1">
+      <c r="A34" s="13" t="str">
+        <v>LAW</v>
+      </c>
+      <c r="B34" s="15" t="str">
+        <v>Fordham Ancient History Sourcebook — Code of Hammurabi, L. W. King translation</v>
+      </c>
+      <c r="C34" s="13" t="str">
+        <v>Numbered laws 8 and 48 only; original eighteenth century BCE, modern English translation. Do not use the dated introductory commentary as the factual key.</v>
+      </c>
+      <c r="D34" s="13" t="str">
+        <v>Translation selected. Prepare short attributed accessible versions and pair with object/context evidence in Step 6.</v>
+      </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2865,45 +2877,39 @@
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="6" t="str">
+    <row r="36">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="6" t="str">
         <v>Recovered learning assignments</v>
       </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-    </row>
-    <row r="37" ht="55" customHeight="1">
-      <c r="A37" s="9" t="str">
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="9" t="str">
         <v>Assignment</v>
       </c>
-      <c r="B37" s="9" t="str">
+      <c r="B38" s="9" t="str">
         <v>Local recovered IDs</v>
       </c>
-      <c r="C37" s="9" t="str">
+      <c r="C38" s="9" t="str">
         <v>Use</v>
-      </c>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-    </row>
-    <row r="38" ht="60" customHeight="1">
-      <c r="A38" s="11" t="str">
-        <v>Home</v>
-      </c>
-      <c r="B38" s="11" t="str">
-        <v>SS.01, SS.02, SS.03, SS.04, SS.05, SS.06, SS.07, SS.08, SS.09, SS.10</v>
-      </c>
-      <c r="C38" s="11" t="str">
-        <v>Historical bundled learning retained; not official national or Tennessee codes.</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -2913,14 +2919,14 @@
       <c r="I38" s="3"/>
     </row>
     <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="13" t="str">
-        <v>Recurrence</v>
-      </c>
-      <c r="B39" s="13" t="str">
-        <v>Prior-grade foundations</v>
-      </c>
-      <c r="C39" s="13" t="str">
-        <v>SSP.01–06 recur across the term. Course appendix contains the official TN content check.</v>
+      <c r="A39" s="11" t="str">
+        <v>Home</v>
+      </c>
+      <c r="B39" s="11" t="str">
+        <v>SS.01, SS.02, SS.03, SS.04, SS.05, SS.06, SS.07, SS.08, SS.09, SS.10</v>
+      </c>
+      <c r="C39" s="11" t="str">
+        <v>Historical bundled learning retained; not official national or Tennessee codes.</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
@@ -2929,10 +2935,16 @@
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
     </row>
-    <row r="40">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="13" t="str">
+        <v>Recurrence</v>
+      </c>
+      <c r="B40" s="13" t="str">
+        <v>Prior-grade foundations</v>
+      </c>
+      <c r="C40" s="13" t="str">
+        <v>SSP.01–06 recur across the term. Course appendix contains the official TN content check.</v>
+      </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -3607,7 +3619,7 @@
     <mergeCell ref="C4:I4"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A29:I29"/>
-    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A37:I37"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C7" r:id="historyLink0"/>
@@ -3621,6 +3633,7 @@
     <hyperlink ref="B31" r:id="historyLink8"/>
     <hyperlink ref="B32" r:id="historyLink9"/>
     <hyperlink ref="B33" r:id="historyLink10"/>
+    <hyperlink ref="B34" r:id="historyLink11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3678,11 +3691,11 @@
     </row>
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="3" t="str">
-        <v>Step 4 block outlines</v>
+        <v>Step 5 teacher plans</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="str">
-        <v>Detailed procedures, exact source excerpts, examples and assessment prompts remain Step 5 work.</v>
+        <v>Full procedures, worked examples, private prompts and clocks in linked plans; Step 6 packets and trials remain.</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -3731,7 +3744,7 @@
         <v>Standards - national</v>
       </c>
     </row>
-    <row r="7" ht="172" customHeight="1">
+    <row r="7" ht="200" customHeight="1">
       <c r="A7" s="16" t="str">
         <v>H2-W1-I
 Week 1 | Individual</v>
@@ -3742,26 +3755,27 @@
       </c>
       <c r="C7" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Egyptian Art
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 3.3 Ancient Egypt: geography, agriculture, religion and society, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D7" s="11" t="str">
-        <v>Model Nile direction versus Upper/Lower labels; connect calendar/irrigation decisions and social work to environmental conditions.</v>
+        <v>Model Nile direction versus Upper/Lower labels; connect calendar/irrigation decisions and social work to environmental conditions. Example: Upper Egypt lies upstream toward the south; river direction and north are different concepts. Calendar knowledge helps plan work but cannot guarantee harvests; occupations depend on institutions as well as the river.</v>
       </c>
       <c r="E7" s="11" t="str">
-        <v>Annotate map and seasonal sequence; compare occupation roles; add a respectful beliefs/context caption.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate map and seasonal sequence; compare occupation roles; add a respectful beliefs/context caption. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F7" s="11" t="str">
         <v>Collect: Individual map plus one agriculture/institution explanation and belief-context annotation.
-Judge: Correct relative locations; causal links use evidence; afterlife belief is attributed to historical practitioners.
-Feedback/support: If Upper means north, follow upstream and recheck a blank map; chunk text and read captions together.</v>
+Prompt: Label all seven Egyptian map features from the teacher key. Explain flood/calendar/irrigation decisions and one occupational relationship; attribute an afterlife belief without claiming the belief is independently proven.
+Criteria: Correct relative locations; causal links use evidence; afterlife belief is attributed to historical practitioners.
+Response to difficulty: If Upper means north, follow upstream and recheck a blank map; chunk text and read captions together.</v>
       </c>
       <c r="G7" s="11" t="str">
-        <v>Prepare two brief context cards and exact map/monument records; carry Egypt annotations to W1-G.</v>
+        <v>Prepare two brief context cards and exact map/monument records; carry Egypt annotations to W1-G. Carry saved private evidence and unresolved component notes to H2-W1-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H7" s="11" t="str">
-        <v>Teach / revisit: Egypt map: Nile/delta, Upper/Lower Egypt, Nubia, Sahara, Red/Mediterranean seas; irrigation/calendar; occupations, enslaved people, pharaoh; polytheism, afterlife/mummification.
-Practice: Annotate map and seasonal sequence; compare occupation roles; add a respectful beliefs/context caption.
+        <v>Teach / revisit: Explain Egypt along the Nile
+Practice: source/context reasoning through the project task.
 Check: Individual map plus one agriculture/institution explanation and belief-context annotation.
 Builds on: H1 rivers, institutions and source labels.</v>
       </c>
@@ -3769,7 +3783,7 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.Geo.4.6-8, D2.Civ.6.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T3, T5 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
       </c>
     </row>
     <row r="8" ht="242" customHeight="1">
@@ -3783,26 +3797,27 @@
       </c>
       <c r="C8" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Egyptian Art
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 3.3 Ancient Egypt: rulers and material culture; paired Egypt/Nubia contexts, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D8" s="13" t="str">
-        <v>Model how a later discovery changes an interpretation; give Nubian actors their own context rather than defining them only through Egypt.</v>
+        <v>Model how a later discovery changes an interpretation; give Nubian actors their own context rather than defining them only through Egypt. Example: A monument records an ancient ruler's claim; a modern discovery record dates recovery. Neither dates the other's event. A trade object supports contact without proving peaceful relations in every period.</v>
       </c>
       <c r="E8" s="13" t="str">
-        <v>Build a compact evidence panel; place rulers/discovery on separate timeline lanes; compare trade/conflict accounts and artifact limits. Compare a brief, sourced modern excavator oral recollection with a dated discovery record; distinguish recollection from ancient eyewitness evidence.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Build a compact evidence panel; place rulers/discovery on separate timeline lanes; compare trade/conflict accounts and artifact limits. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F8" s="13" t="str">
-        <v>Collect: Each student explains one figure’s significance, an achievement and how a discovery or perspective changes knowledge. Include one comparison of the oral recollection and discovery record.
-Judge: Distinguishes ancient events from modern excavation; includes Nubian agency and sourced achievement effects.
-Feedback/support: If tomb wealth proves all lives were alike, compare nonelite evidence and recheck; use a discovery/event timeline key.</v>
+        <v>Collect: Each student explains one figure’s significance, an achievement and how a discovery or perspective changes knowledge. Oral/written comparison is collected only after the oral source is verified; otherwise this modality remains Conditional.
+Prompt: Distinguish Hatshepsut's policy, Ramses II's conquest and the modern discovery of Tutankhamun. Explain hieroglyphs, papyrus and Giza's significance. Use one Nubian-perspective clue to qualify a trade/conflict claim.
+Criteria: Distinguishes ancient events from modern excavation; includes Nubian agency and sourced achievement effects.
+Response to difficulty: If tomb wealth proves all lives were alike, compare nonelite evidence and recheck; use a discovery/event timeline key.</v>
       </c>
       <c r="G8" s="13" t="str">
-        <v>Keep panel to existing notes and two captions; select a Nubian-perspective source before Step 5. Select and caption a 60–90-second recorded excavator recollection, or attributed oral-history transcript, with creator/date/context; keep total new reading/listening within the block budget.</v>
+        <v>Keep panel to existing notes and two captions; select a Nubian-perspective source before Step 5. Select and caption a 60–90-second recorded excavator recollection, or attributed oral-history transcript, with creator/date/context; keep total new reading/listening within the block budget. Carry saved private evidence and unresolved component notes to H2-W2-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H8" s="13" t="str">
-        <v>Teach / revisit: Hatshepsut policies/trade, Ramses military growth, Tutankhamun tomb discovery and revised knowledge; hieroglyphics/papyrus/Giza; Nubian trade/conflict and agency.
-Practice: Build a compact evidence panel; place rulers/discovery on separate timeline lanes; compare trade/conflict accounts and artifact limits. Compare a brief, sourced modern excavator oral recollection with a dated discovery record; distinguish recollection from ancient eyewitness evidence.
+        <v>Teach / revisit: Connect Egypt and Nubia
+Practice: source/context reasoning through the project task.
 Check: Each student explains one figure’s significance, an achievement and how a discovery or perspective changes knowledge. Include one comparison of the oral recollection and discovery record.
 Builds on: Egypt map/social structure and H1 evidence limits.</v>
       </c>
@@ -3810,10 +3825,10 @@
         <v>C3 Primary: D2.His.3.6-8, D2.His.6.6-8, D2.His.10.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T8, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="9" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="9" ht="200" customHeight="1">
       <c r="A9" s="16" t="str">
         <v>H2-W2-I
 Week 2 | Individual</v>
@@ -3824,26 +3839,27 @@
       </c>
       <c r="C9" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 4.4 The Hebrews: origin traditions and Judaism, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D9" s="11" t="str">
-        <v>Distinguish traditions recorded in sacred texts, archaeological evidence and modern historical interpretation; teach religions academically with a common template.</v>
+        <v>Distinguish traditions recorded in sacred texts, archaeological evidence and modern historical interpretation; teach religions academically with a common template. Example: A religious narrative supports what a community preserves about origins; a modern historical map is an interpretation. Attribute a movement account and seek independent evidence before asserting a precise route.</v>
       </c>
       <c r="E9" s="11" t="str">
-        <v>Map attributed movement accounts; annotate people/texts/beliefs/context; compare what different source types can establish.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Map attributed movement accounts; annotate people/texts/beliefs/context; compare what different source types can establish. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F9" s="11" t="str">
         <v>Collect: Individual route/source explanation and a respectful Judaism profile.
-Judge: Uses attribution where historical evidence is contested; accurate text/belief terms; no devotional activity required.
-Feedback/support: If every account is called verified eyewitness history, classify source type and recheck; provide pronunciation and neutral profiles.</v>
+Prompt: Locate the six Israel features. Attribute the traditional Ur–Canaan–Egypt account. Complete a Judaism profile naming Abraham, Moses, Tanakh/Torah, monotheism, commandments and ethical responsibility; distinguish tradition from corroborated evidence.
+Criteria: Uses attribution where historical evidence is contested; accurate text/belief terms; no devotional activity required.
+Response to difficulty: If every account is called verified eyewitness history, classify source type and recheck; provide pronunciation and neutral profiles.</v>
       </c>
       <c r="G9" s="11" t="str">
-        <v>Select an accessible religious-studies/history source and exact attributed excerpts.</v>
+        <v>Select an accessible religious-studies/history source and exact attributed excerpts. Carry saved private evidence and unresolved component notes to H2-W2-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H9" s="11" t="str">
-        <v>Teach / revisit: Dead/Red/Mediterranean seas, Jordan, Jerusalem, Sinai; Ur/Canaan/Egypt movements; Judaism, Abraham/Moses, Tanakh/Torah, monotheism, Ten Commandments, responsibility.
-Practice: Map attributed movement accounts; annotate people/texts/beliefs/context; compare what different source types can establish.
+        <v>Teach / revisit: Trace ancient Israel and its traditions
+Practice: source/context reasoning through the project task.
 Check: Individual route/source explanation and a respectful Judaism profile.
 Builds on: Chronology, geography and source-purpose reasoning.</v>
       </c>
@@ -3851,10 +3867,10 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.His.4.6-8, D3.2.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T2, T3 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="10" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="10" ht="200" customHeight="1">
       <c r="A10" s="17" t="str">
         <v>H2-W2-G
 Week 2 | Group</v>
@@ -3865,26 +3881,27 @@
       </c>
       <c r="C10" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Egyptian Art
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 4.4 The Hebrews: kingdoms, conquest, exile and return, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D10" s="13" t="str">
-        <v>Model a dated movement explanation separating political cause from a tradition’s meaning; avoid modern-border substitution.</v>
+        <v>Model a dated movement explanation separating political cause from a tradition’s meaning; avoid modern-border substitution. Example: Compare a different conquest sequence: conquest can change rulers, cause displacement and later permit returns under another empire. Return does not mean every displaced family returned.</v>
       </c>
       <c r="E10" s="13" t="str">
-        <v>Construct kingdom/conquest sequence; compare one Egypt/Nubia and Israel movement; add two evidence-based exhibit captions.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Construct kingdom/conquest sequence; compare one Egypt/Nubia and Israel movement; add two evidence-based exhibit captions. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F10" s="13" t="str">
         <v>Collect: Private cause/effect sequence and comparison with dated evidence from both contexts.
-Judge: Actors/sequence are coherent; multiple political/geographic factors appear; similarity does not erase difference.
-Feedback/support: If all exile periods merge, separate timeline bands and recheck events; use a movement legend.</v>
+Prompt: Sequence Saul, David, Solomon, Assyrian/Babylonian conquest, exile and Persian return. Explain political causes and compare one movement with Egypt/Nubia using a similarity, a difference and dated evidence.
+Criteria: Actors/sequence are coherent; multiple political/geographic factors appear; similarity does not erase difference.
+Response to difficulty: If all exile periods merge, separate timeline bands and recheck events; use a movement legend.</v>
       </c>
       <c r="G10" s="13" t="str">
-        <v>Limit captions to 60–80 words each; retain Israel panel and shared chronology.</v>
+        <v>Limit captions to 60–80 words each; retain Israel panel and shared chronology. Carry saved private evidence and unresolved component notes to H2-W3-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H10" s="13" t="str">
-        <v>Teach / revisit: Saul, David/Jerusalem, Solomon/temple; kingdom division, Assyrian/Babylonian conquest/exiles, Persian return; cross-society comparison.
-Practice: Construct kingdom/conquest sequence; compare one Egypt/Nubia and Israel movement; add two evidence-based exhibit captions.
+        <v>Teach / revisit: Explain kingdoms, exile and return
+Practice: source/context reasoning through the project task.
 Check: Private cause/effect sequence and comparison with dated evidence from both contexts.
 Builds on: Israel routes/traditions and Egypt/Nubia evidence.</v>
       </c>
@@ -3892,10 +3909,10 @@
         <v>C3 Primary: D2.His.1.6-8, D2.His.14.6-8, D4.2.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T5, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="11" ht="144" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="11" ht="200" customHeight="1">
       <c r="A11" s="16" t="str">
         <v>H2-W3-I
 Week 3 | Individual</v>
@@ -3906,26 +3923,27 @@
       </c>
       <c r="C11" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 5.4 Vedic India to the Fall of the Maurya Empire: Indus cities and geographic context, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D11" s="11" t="str">
-        <v>Model a city-plan inference and its limits; compare economic/environmental decisions without claiming undeciphered writing supplies a known government.</v>
+        <v>Model a city-plan inference and its limits; compare economic/environmental decisions without claiming undeciphered writing supplies a known government. Example: A hypothetical city plan shows drains and regular streets. These support organized construction, but cannot name its rulers or prove all houses had equal access.</v>
       </c>
       <c r="E11" s="11" t="str">
-        <v>Annotate map/city plan; identify water/sanitation evidence; compare a useful Mesopotamian pattern with a distinct Indus case.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate map/city plan; identify water/sanitation evidence; compare a useful Mesopotamian pattern with a distinct Indus case. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F11" s="11" t="str">
         <v>Collect: Individual plan-based inference and explanation of two documented achievements.
-Judge: Separates observation from unknown institutions; explains infrastructure rather than praising advanced design alone.
-Feedback/support: If a regular grid proves democracy, show inference limits and recheck a different plan; use magnified plans.</v>
+Prompt: Label India's six features and explain monsoon effects. Use the Indus plan to explain grid, bricks and sanitation. Compare with Mesopotamia and state what a street plan cannot establish about rulers or religion.
+Criteria: Separates observation from unknown institutions; explains infrastructure rather than praising advanced design alone.
+Response to difficulty: If a regular grid proves democracy, show inference limits and recheck a different plan; use magnified plans.</v>
       </c>
       <c r="G11" s="11" t="str">
-        <v>Prepare dated archaeological plan/source card and retain inference notes for India panel.</v>
+        <v>Prepare dated archaeological plan/source card and retain inference notes for India panel. Carry saved private evidence and unresolved component notes to H2-W3-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H11" s="11" t="str">
-        <v>Teach / revisit: India subcontinent, Himalayas, Indus/Ganges, Indian Ocean, monsoons; Harappa/Mohenjo-Daro, bricks, grid roads and sanitation.
-Practice: Annotate map/city plan; identify water/sanitation evidence; compare a useful Mesopotamian pattern with a distinct Indus case.
+        <v>Teach / revisit: Investigate Indus cities
+Practice: source/context reasoning through the project task.
 Check: Individual plan-based inference and explanation of two documented achievements.
 Builds on: H1 city systems and H2 maps.</v>
       </c>
@@ -3933,7 +3951,7 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.Geo.4.6-8, D2.His.9.6-8
 Supporting: D3.1.6-8
 NCSS themes: T3, T7, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
       </c>
     </row>
     <row r="12" ht="214" customHeight="1">
@@ -3947,26 +3965,27 @@
       </c>
       <c r="C12" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 5.4 Vedic India to the Fall of the Maurya Empire: Vedic society, Hinduism and Buddhism, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D12" s="13" t="str">
-        <v>Use matched neutral religion profiles; distinguish beliefs, social practices and later developments. Explain changing scholarship on migration rather than a single unqualified invasion story.</v>
+        <v>Use matched neutral religion profiles; distinguish beliefs, social practices and later developments. Explain changing scholarship on migration rather than a single unqualified invasion story. Example: A matched profile separates Hindu moksha and Buddhist nirvana without treating them as identical. A later numeral record illustrates chronological separation from an earlier city plan.</v>
       </c>
       <c r="E12" s="13" t="str">
-        <v>Compare the two profiles and dated evidence cards; explain hierarchy’s daily-life effects; attach a short achievement timeline.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Compare the two profiles and dated evidence cards; explain hierarchy’s daily-life effects; attach a short achievement timeline. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F12" s="13" t="str">
         <v>Collect: Private comparison including people/texts/beliefs, a social-position explanation and correctly dated achievement.
-Judge: Keeps traditions distinct and attributed; does not portray caste or either religion as uniform across all people/time.
-Feedback/support: If unfamiliar terms replace explanation, model one in context and recheck another; provide a glossary and reduced-copy organizer.</v>
+Prompt: Compare Hinduism and Buddhism using people/texts, goals and beliefs. Explain Aryan migration/language and hierarchy with a bounded daily-life example. Date medicine/yoga/numerals separately from Indus urbanism; do not assign all achievements to one era.
+Criteria: Keeps traditions distinct and attributed; does not portray caste or either religion as uniform across all people/time.
+Response to difficulty: If unfamiliar terms replace explanation, model one in context and recheck another; provide a glossary and reduced-copy organizer.</v>
       </c>
       <c r="G12" s="13" t="str">
-        <v>Busiest H2 block: two profiles totaling about 250 words plus a diagram. Verify comprehension/time; move caption polish to W4-I, never required reading to homework.</v>
+        <v>Busiest H2 block: two profiles totaling about 250 words plus a diagram. Verify comprehension/time; move caption polish to W4-I, never required reading to homework. Carry saved private evidence and unresolved component notes to H2-W4-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H12" s="13" t="str">
-        <v>Teach / revisit: Indo-Aryan migrations/language/religious change; caste/social hierarchy; Hinduism: Vedas, dharma/karma/reincarnation/moksha; Buddhism: Siddhartha, Tripitaka, Four Noble Truths/Eightfold Path/Nirvana; medicine, yoga and numerals with correct dates.
-Practice: Compare the two profiles and dated evidence cards; explain hierarchy’s daily-life effects; attach a short achievement timeline.
+        <v>Teach / revisit: Explain traditions and social change in India
+Practice: source/context reasoning through the project task.
 Check: Private comparison including people/texts/beliefs, a social-position explanation and correctly dated achievement.
 Builds on: Institution/perspective reasoning and Indus chronology.</v>
       </c>
@@ -3974,10 +3993,10 @@
         <v>C3 Primary: D2.His.4.6-8, D2.Civ.6.6-8, D3.3.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T4, T5, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="13" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="13" ht="214" customHeight="1">
       <c r="A13" s="16" t="str">
         <v>H2-W4-I
 Week 4 | Individual</v>
@@ -3988,26 +4007,27 @@
       </c>
       <c r="C13" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Egyptian Art
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from Reuse three H2 society profiles, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D13" s="11" t="str">
-        <v>Model comparison from two explicit pieces of evidence, with a counterexample and source limitation.</v>
+        <v>Model comparison from two explicit pieces of evidence, with a counterexample and source limitation. Example: Compare Nile irrigation and Indus drainage through purpose, evidence and limits. Both manage water; their distinct environmental problems prevent a single identical explanation.</v>
       </c>
       <c r="E13" s="11" t="str">
-        <v>Use a targeted retrieval clinic; finish three short panels from saved notes; individually compare two societies and respond to a third-society question.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Use a targeted retrieval clinic; finish three short panels from saved notes; individually compare two societies and respond to a third-society question. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F13" s="11" t="str">
         <v>Collect: Independent comparison plus all-three-society retrieval record and one revised claim.
-Judge: No society omitted; claims use common dimensions and context-specific evidence; revision improves reasoning.
-Feedback/support: If team specialization hides missing learning, administer short private checks and targeted source review; extend by challenging a comparison.</v>
+Prompt: Compare two societies using geography and institutions, citing one source each. Answer the teacher's third-society question. Show one evidence-based correction in the three-panel atlas and explain its importance.
+Criteria: No society omitted; claims use common dimensions and context-specific evidence; revision improves reasoning.
+Response to difficulty: If team specialization hides missing learning, administer short private checks and targeted source review; extend by challenging a comparison.</v>
       </c>
       <c r="G13" s="11" t="str">
-        <v>Keep one atlas, no separate long essays; prepare fresh map/source mini-checks for W4-G.</v>
+        <v>Keep one atlas, no separate long essays; prepare fresh map/source mini-checks for W4-G. Carry saved private evidence and unresolved component notes to H2-W4-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H13" s="11" t="str">
-        <v>Teach / revisit: Common geographic, institutional and belief questions; Egypt/Nubia, Israel and India each required.
-Practice: Use a targeted retrieval clinic; finish three short panels from saved notes; individually compare two societies and respond to a third-society question.
+        <v>Teach / revisit: Compare all three society panels
+Practice: source/context reasoning through the project task.
 Check: Independent comparison plus all-three-society retrieval record and one revised claim.
 Builds on: All H2 notes, profiles, maps and chronology.</v>
       </c>
@@ -4015,10 +4035,10 @@
         <v>C3 Primary: D2.His.16.6-8, D4.1.6-8, D4.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T3, T5, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="14" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="14" ht="214" customHeight="1">
       <c r="A14" s="17" t="str">
         <v>H2-W4-G
 Week 4 | Group</v>
@@ -4029,26 +4049,27 @@
       </c>
       <c r="C14" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Egyptian Art
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from Held-back map/context; reuse three profiles, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D14" s="13" t="str">
-        <v>Model audience questions about evidence and coherent explanation, not costume or visual polish.</v>
+        <v>Model audience questions about evidence and coherent explanation, not costume or visual polish. Example: A new regional map locates contact, but lacks a trade object's maker or journey. Revise an overconfident route caption to an evidenced possibility.</v>
       </c>
       <c r="E14" s="13" t="str">
-        <v>Six short team walkthroughs; every learner explains a source; collect a fresh map/context response and revise one caption.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Six short team walkthroughs; every learner explains a source; collect a fresh map/context response and revise one caption. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F14" s="13" t="str">
         <v>Collect: Teacher-observed explanation and private fresh source/map interpretation; shared atlas assessed separately.
-Judge: Accurate context/source use; all required societies remain represented; feedback changes a claim or connection.
-Feedback/support: If a comparison overgeneralizes belief, require attribution and a new example; record unresolved society/component for H3 opening.</v>
+Prompt: Explain one source for each atlas society. Interpret a fresh dated map/context card: locate its setting, make a supported claim and identify a limitation. Revise one caption; keep your private response separate from the team atlas.
+Criteria: Accurate context/source use; all required societies remain represented; feedback changes a claim or connection.
+Response to difficulty: If a comparison overgeneralizes belief, require attribution and a new example; record unresolved society/component for H3 opening.</v>
       </c>
       <c r="G14" s="13" t="str">
-        <v>Archive individual checks separately; carry comparison and scholarly uncertainty routines into H3.</v>
+        <v>Archive individual checks separately; carry comparison and scholarly uncertainty routines into H3. Carry saved private evidence and unresolved component notes to H3-W1-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H14" s="13" t="str">
-        <v>Teach / revisit: Walkthrough, individual fresh map/source application and feedback.
-Practice: Six short team walkthroughs; every learner explains a source; collect a fresh map/context response and revise one caption.
+        <v>Teach / revisit: Defend the linked atlas exhibit
+Practice: source/context reasoning through the project task.
 Check: Teacher-observed explanation and private fresh source/map interpretation; shared atlas assessed separately.
 Builds on: Evidence-based comparison and source limitations.</v>
       </c>
@@ -4056,7 +4077,7 @@
         <v>C3 Primary: D4.2.6-8, D4.5.6-8, D3.2.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
       </c>
     </row>
     <row r="15">
@@ -4113,7 +4134,7 @@
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
     </row>
-    <row r="19" ht="102" customHeight="1">
+    <row r="19" ht="116" customHeight="1">
       <c r="A19" s="11" t="str">
         <v>H2-W1-I</v>
       </c>
@@ -4125,7 +4146,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D19" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -4133,19 +4154,19 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" ht="130" customHeight="1">
+    <row r="20" ht="158" customHeight="1">
       <c r="A20" s="13" t="str">
         <v>H2-W1-G</v>
       </c>
       <c r="B20" s="13" t="str">
         <v>D2.His.3.6-8, D2.His.6.6-8, D2.His.10.6-8
-Each student explains one figure’s significance, an achievement and how a discovery or perspective changes knowledge. Include one comparison of the oral recollection and discovery record.</v>
+Each student explains one figure’s significance, an achievement and how a discovery or perspective changes knowledge. Oral/written comparison is collected only after the oral source is verified; otherwise this modality remains Conditional.</v>
       </c>
       <c r="C20" s="13" t="str">
         <v>D3.1.6-8</v>
       </c>
       <c r="D20" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -4153,7 +4174,7 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" ht="102" customHeight="1">
+    <row r="21" ht="116" customHeight="1">
       <c r="A21" s="11" t="str">
         <v>H2-W2-I</v>
       </c>
@@ -4165,7 +4186,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D21" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -4173,7 +4194,7 @@
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" ht="102" customHeight="1">
+    <row r="22" ht="116" customHeight="1">
       <c r="A22" s="13" t="str">
         <v>H2-W2-G</v>
       </c>
@@ -4185,7 +4206,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D22" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -4193,7 +4214,7 @@
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" ht="102" customHeight="1">
+    <row r="23" ht="116" customHeight="1">
       <c r="A23" s="11" t="str">
         <v>H2-W3-I</v>
       </c>
@@ -4205,7 +4226,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D23" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -4213,7 +4234,7 @@
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
     </row>
-    <row r="24" ht="102" customHeight="1">
+    <row r="24" ht="116" customHeight="1">
       <c r="A24" s="13" t="str">
         <v>H2-W3-G</v>
       </c>
@@ -4225,7 +4246,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D24" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -4233,7 +4254,7 @@
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
     </row>
-    <row r="25" ht="102" customHeight="1">
+    <row r="25" ht="116" customHeight="1">
       <c r="A25" s="11" t="str">
         <v>H2-W4-I</v>
       </c>
@@ -4245,7 +4266,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D25" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -4253,7 +4274,7 @@
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
     </row>
-    <row r="26" ht="102" customHeight="1">
+    <row r="26" ht="116" customHeight="1">
       <c r="A26" s="13" t="str">
         <v>H2-W4-G</v>
       </c>
@@ -4265,7 +4286,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D26" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -4329,7 +4350,7 @@
     </row>
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="11" t="str">
-        <v>Project outline</v>
+        <v>Detailed project plan</v>
       </c>
       <c r="B31" s="14" t="str">
         <v>H2 River Kingdoms Atlas</v>
@@ -4338,7 +4359,7 @@
         <v>One shared atlas exhibit with three concise society panels and a common timeline/map. Every student completes evidence for all three; no specialist-only coverage.</v>
       </c>
       <c r="D31" s="11" t="str">
-        <v>Step 4 outline exists; detailed Step 5 lessons pending.</v>
+        <v>Eight detailed Step 5 plans developed; Step 6 materials remain.</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -4357,7 +4378,7 @@
         <v>Teacher background: early humans, river-valley societies, ancient Israel/India/China/Greece/Rome. Select topic sections and primary-source boxes; prepare short attributed student adaptations.</v>
       </c>
       <c r="D32" s="13" t="str">
-        <v>Teacher reference located; exact excerpts, dates, image rights, reading fit and source packets remain Step 5/6 work. Do not assign whole college chapters.</v>
+        <v>Named section selections specified in all 32 detailed plans. Bounded Grade 6 adaptations and source boxes remain Step 6; do not assign whole college chapters.</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -5219,11 +5240,11 @@
     </row>
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="3" t="str">
-        <v>Step 4 block outlines</v>
+        <v>Step 5 teacher plans</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="str">
-        <v>Detailed procedures, exact source excerpts, examples and assessment prompts remain Step 5 work.</v>
+        <v>Full procedures, worked examples, private prompts and clocks in linked plans; Step 6 packets and trials remain.</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -5272,7 +5293,7 @@
         <v>Standards - national</v>
       </c>
     </row>
-    <row r="7" ht="158" customHeight="1">
+    <row r="7" ht="200" customHeight="1">
       <c r="A7" s="16" t="str">
         <v>H3-W1-I
 Week 1 | Individual</v>
@@ -5283,26 +5304,27 @@
       </c>
       <c r="C7" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 5.1 Ancient China: early dynasties, geography and Zhou authority, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D7" s="11" t="str">
-        <v>Model a geographic governance explanation; distinguish traditional accounts of Xia from excavated Shang evidence.</v>
+        <v>Model a geographic governance explanation; distinguish traditional accounts of Xia from excavated Shang evidence. Example: Shang material records and Xia traditions offer different evidence conditions. Mountains can constrain routes while exchange still occurs; geography influences possibilities without dictating one government.</v>
       </c>
       <c r="E7" s="11" t="str">
-        <v>Annotate map and dynasty sequence; explain authority claims and Legalist responses to governing challenges; start China panel.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate map and dynasty sequence; explain authority claims and Legalist responses to governing challenges; start China panel. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F7" s="11" t="str">
         <v>Collect: Individual map/context explanation and one claim distinguishing tradition/evidence.
-Judge: Maps all required features; connects geography to institutions without assuming total isolation; dates/claim types are explicit.
-Feedback/support: If dynasty names become a list, connect a challenge and response then recheck; use a labeled timeline strip.</v>
+Prompt: Label China's six features and sequence Xia tradition, Shang evidence and Zhou authority. Explain one geographic influence without claiming complete isolation. Contrast Mandate of Heaven and Legalism as governing ideas.
+Criteria: Maps all required features; connects geography to institutions without assuming total isolation; dates/claim types are explicit.
+Response to difficulty: If dynasty names become a list, connect a challenge and response then recheck; use a labeled timeline strip.</v>
       </c>
       <c r="G7" s="11" t="str">
-        <v>Prepare two context cards and retain authority questions for Qin/Han.</v>
+        <v>Prepare two context cards and retain authority questions for Qin/Han. Carry saved private evidence and unresolved component notes to H3-W1-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H7" s="11" t="str">
-        <v>Teach / revisit: Gobi, Himalayas, Pacific, Tibet plateau, Yangtze/Yellow rivers; Xia tradition and Shang evidence; geographic governing constraints; Zhou/Mandate of Heaven and Legalism.
-Practice: Annotate map and dynasty sequence; explain authority claims and Legalist responses to governing challenges; start China panel.
+        <v>Teach / revisit: Locate China and explain early authority
+Practice: source/context reasoning through the project task.
 Check: Individual map/context explanation and one claim distinguishing tradition/evidence.
 Builds on: H1/H2 geography, evidence and hierarchy.</v>
       </c>
@@ -5310,10 +5332,10 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.His.1.6-8, D2.Civ.6.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T3, T6 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="8" ht="200" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="8" ht="256" customHeight="1">
       <c r="A8" s="17" t="str">
         <v>H3-W1-G
 Week 1 | Group</v>
@@ -5324,26 +5346,27 @@
       </c>
       <c r="C8" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Han Dynasty (206 BCE–220 CE); British Library / International Dunhuang Programme — Diamond Sutra display guide
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 5.1 Ancient China: Qin/Han and Confucian institutions; Met Han essay, government and timekeeping paragraphs, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D8" s="13" t="str">
-        <v>Compare a philosophy excerpt and institutional account; show a dated invention strip rather than putting every Chinese invention in Han.</v>
+        <v>Compare a philosophy excerpt and institutional account; show a dated invention strip rather than putting every Chinese invention in Han. Example: A dated later printing example cannot automatically be Han because it is Chinese. Distinguish a earliest surviving record from an invention date; a text praising order does not prove universal social agreement.</v>
       </c>
       <c r="E8" s="13" t="str">
-        <v>Trace policy/institution links; annotate Han timekeeping/astronomy, paper/silk/seismograph evidence; place compass, porcelain and printing records in evidenced periods.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Trace policy/institution links; annotate Han timekeeping/astronomy, paper/silk/seismograph evidence; place compass, porcelain and printing records in evidenced periods. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F8" s="13" t="str">
         <v>Collect: Each student explains institutional influence and corrects one unsupported invention/date attribution.
-Judge: Connects Confucian ideas to institutions; distinguishes invention, surviving evidence and later use. TN 6.39 chronology remains flagged.
-Feedback/support: If latest evidence becomes earliest invention, model the distinction and recheck; provide a date/evidence grid.</v>
+Prompt: Explain Qin unification/standardization and Confucius/Analects/kinship/order; connect a Han institution to Confucian ideas. Classify paper, silk, seismograph, compass, porcelain and printing claims by evidence/date; reject unsupported Han printing attribution.
+Criteria: Connects Confucian ideas to institutions; distinguishes invention, surviving evidence and later use. TN 6.39 chronology remains flagged.
+Response to difficulty: If latest evidence becomes earliest invention, model the distinction and recheck; provide a date/evidence grid.</v>
       </c>
       <c r="G8" s="13" t="str">
-        <v>Verify all technology dates and exact source excerpts. Do not teach woodblock printing as securely Han; resolve the TN wording concern with the school.</v>
+        <v>Verify all technology dates and exact source excerpts. Do not teach woodblock printing as securely Han; resolve the TN wording concern with the school. Carry saved private evidence and unresolved component notes to H3-W2-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H8" s="13" t="str">
-        <v>Teach / revisit: Qin Shi Huangdi/unification, walls/roads/canals/writing; Confucius, Analects, kinship/order/hierarchy; Han government and technological achievement chronology.
-Practice: Trace policy/institution links; annotate Han timekeeping/astronomy, paper/silk/seismograph evidence; place compass, porcelain and printing records in evidenced periods.
+        <v>Teach / revisit: Connect Qin, Confucius and Han institutions
+Practice: source/context reasoning through the project task.
 Check: Each student explains institutional influence and corrects one unsupported invention/date attribution.
 Builds on: China authority sequence and source limitation routines.</v>
       </c>
@@ -5351,10 +5374,10 @@
         <v>C3 Primary: D2.Civ.6.6-8, D2.His.4.6-8, D2.His.10.6-8
 Supporting: D3.1.6-8
 NCSS themes: T4, T5, T6, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="9" ht="186" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="9" ht="214" customHeight="1">
       <c r="A9" s="16" t="str">
         <v>H3-W2-I
 Week 2 | Individual</v>
@@ -5364,27 +5387,28 @@
 Aegean, Asia Minor, Athens, Macedonia, Mediterranean, Peloponnese, Sparta; mountains/sea, city-states/trade/colonies; polis, law, civic participation; Athens/Sparta government, education, women and enslaved people.</v>
       </c>
       <c r="C9" s="14" t="str">
-        <v>OpenStax — World History Volume 1, to 1500; American School of Classical Studies at Athens — An Athenian Clepsydra
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+        <v>OpenStax — World History Volume 1, to 1500; University of St Andrews MacTutor — Timekeeping in the Ancient World: Water-clocks
+In class: 150–250 words of attributed teacher adaptation from 6.2 Ancient Greece: geography and polis comparison, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D9" s="11" t="str">
-        <v>Model democratic participation with its historical exclusions; compare the same institutional dimensions for Athens and Sparta.</v>
+        <v>Model democratic participation with its historical exclusions; compare the same institutional dimensions for Athens and Sparta. Example: Timed courtroom speaking can regulate participation, yet eligibility still excludes many people. Compare who could speak and who could hold power before applying the word democracy.</v>
       </c>
       <c r="E9" s="11" t="str">
-        <v>Annotate map; build a rights/roles matrix and explain a geographic/economic influence; connect court timing to participation.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate map; build a rights/roles matrix and explain a geographic/economic influence; connect court timing to participation. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F9" s="11" t="str">
         <v>Collect: Private map and citizenship comparison with two institutional differences and an exclusion.
-Judge: No ancient/modern democracy equivalence; group status and place/date shape experiences; map explains spatial pattern.
-Feedback/support: If all residents become citizens, use eligibility/source clinic and recheck; provide matching comparison headings.</v>
+Prompt: Label seven Greek features. Compare Athens and Sparta in government, education and eligible participation, including women and enslaved people. Explain a mountain/sea influence and how timed speaking can shape participation.
+Criteria: No ancient/modern democracy equivalence; group status and place/date shape experiences; map explains spatial pattern.
+Response to difficulty: If all residents become citizens, use eligibility/source clinic and recheck; provide matching comparison headings.</v>
       </c>
       <c r="G9" s="11" t="str">
-        <v>Prepare short context profiles and accessible court-clock source. CLOCK full-text access is conditional; replace with verified equivalent if unavailable.</v>
+        <v>Prepare short context profiles and accessible court-clock source. CLOCK full-text access is conditional; replace with verified equivalent if unavailable. Carry saved private evidence and unresolved component notes to H3-W2-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H9" s="11" t="str">
-        <v>Teach / revisit: Aegean, Asia Minor, Athens, Macedonia, Mediterranean, Peloponnese, Sparta; mountains/sea, city-states/trade/colonies; polis, law, civic participation; Athens/Sparta government, education, women and enslaved people.
-Practice: Annotate map; build a rights/roles matrix and explain a geographic/economic influence; connect court timing to participation.
+        <v>Teach / revisit: Compare Greek places and citizenship
+Practice: source/context reasoning through the project task.
 Check: Private map and citizenship comparison with two institutional differences and an exclusion.
 Builds on: China institutions and H2 common comparison questions.</v>
       </c>
@@ -5392,10 +5416,10 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.Civ.6.6-8, D2.His.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T3, T4, T5, T6, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="10" ht="186" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="10" ht="228" customHeight="1">
       <c r="A10" s="17" t="str">
         <v>H3-W2-G
 Week 2 | Group</v>
@@ -5406,26 +5430,27 @@
       </c>
       <c r="C10" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; Science Museum — Ancient Greek Computing
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 6.2 Ancient Greece: wars and classical ideas; 6.3 The Hellenistic Era: Alexander and diffusion, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D10" s="13" t="str">
-        <v>Separate the two wars on a timeline; use a short philosophy/source example to show context and method, not a claim that all Greeks thought alike.</v>
+        <v>Separate the two wars on a timeline; use a short philosophy/source example to show context and method, not a claim that all Greeks thought alike. Example: A later Hellenistic mechanism predicts celestial cycles; this supports a bounded calculation claim. It does not prove ordinary ships navigated with it or every Greek possessed one.</v>
       </c>
       <c r="E10" s="13" t="str">
-        <v>Complete conflict cause/effect strips; compare three philosopher question cards; add belief/architecture/context notes and inspect astronomical-prediction evidence.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Complete conflict cause/effect strips; compare three philosopher question cards; add belief/architecture/context notes and inspect astronomical-prediction evidence. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F10" s="13" t="str">
         <v>Collect: Individual war comparison and an achievement/significance explanation citing a source limit.
-Judge: Distinct war causes/consequences; philosophers and institutions contextualized; sky models described as historical interpretations.
-Feedback/support: If science lens displaces government/conflict, use private retrieval before adding instrument detail; glossary and comparison cards support reading.</v>
+Prompt: Distinguish Persian and Peloponnesian conflicts and their consequences. Connect Socrates, Plato and Aristotle to different questions. Explain Zeus/Olympics and columns/Parthenon/Acropolis; date Alexander and Hellenistic diffusion and qualify an astronomical-mechanism claim.
+Criteria: Distinct war causes/consequences; philosophers and institutions contextualized; sky models described as historical interpretations.
+Response to difficulty: If science lens displaces government/conflict, use private retrieval before adding instrument detail; glossary and comparison cards support reading.</v>
       </c>
       <c r="G10" s="13" t="str">
-        <v>Busiest H3 pair: cap new prose, reuse timeline, prioritize history evidence; complex gear reconstruction is not planned. Exact Antikythera dates/source boundaries pending.</v>
+        <v>Busiest H3 pair: cap new prose, reuse timeline, prioritize history evidence; complex gear reconstruction is not planned. Exact Antikythera dates/source boundaries pending. Carry saved private evidence and unresolved component notes to H3-W3-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H10" s="13" t="str">
-        <v>Teach / revisit: Persian/Peloponnesian wars causes/effects; polytheism/Olympics; Socrates/Plato/Aristotle and education; Parthenon/Acropolis/columns; Greek/Hellenistic sky observation.
-Practice: Complete conflict cause/effect strips; compare three philosopher question cards; add belief/architecture/context notes and inspect astronomical-prediction evidence.
+        <v>Teach / revisit: Explain Greek conflict, ideas and achievements
+Practice: source/context reasoning through the project task.
 Check: Individual war comparison and an achievement/significance explanation citing a source limit.
 Builds on: Greek map/citizenship and China science context.</v>
       </c>
@@ -5433,10 +5458,10 @@
         <v>C3 Primary: D2.His.14.6-8, D2.His.3.6-8, D2.His.6.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T2, T5, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="11" ht="186" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="11" ht="256" customHeight="1">
       <c r="A11" s="16" t="str">
         <v>H3-W3-I
 Week 3 | Individual</v>
@@ -5446,27 +5471,28 @@
 Han water clocks/sundials, Athenian court timer, astronomical patterns; elapsed-time versus time-of-day; historical evidence versus modern measurement.</v>
       </c>
       <c r="C11" s="14" t="str">
-        <v>The Met — Han Dynasty (206 BCE–220 CE); American School of Classical Studies at Athens — An Athenian Clepsydra; Science Museum — Ancient Greek Computing
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+        <v>The Met — Han Dynasty (206 BCE–220 CE); University of St Andrews MacTutor — Timekeeping in the Ancient World: Water-clocks; Science Museum — Ancient Greek Computing
+In class: 150–250 words of attributed teacher adaptation from MacTutor Water-clocks: opening through Athenian courts and flow/pressure explanation; Met Han timekeeping paragraph, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D11" s="11" t="str">
-        <v>Model a source-purpose comparison and one controlled water-timer plan; supplied dated shadow observations illustrate a different method.</v>
+        <v>Model a source-purpose comparison and one controlled water-timer plan; supplied dated shadow observations illustrate a different method. Example: Illustrative repeats of 32, 35 and 33 seconds have a 3-second range. Fixing start level helps comparison; a replica cannot independently establish an ancient device's accuracy.</v>
       </c>
       <c r="E11" s="11" t="str">
-        <v>Select historical evidence from both societies; define elapsed-time question, fixed vessel/hole/start volume and repeated observations; predict limitations; read supplied shadow table.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Select historical evidence from both societies; define elapsed-time question, fixed vessel/hole/start volume and repeated observations; predict limitations; read supplied shadow table. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F11" s="11" t="str">
         <v>Collect: Individual comparison plan naming sources, measurements/units, controls and evidence limits.
-Judge: Same comparison questions for both cases; no direct China–Greece transmission claim; modern model is labeled.
-Feedback/support: If timer is mistaken for navigation proof, identify its documented use and recheck; offer a protocol diagram without filling in reasoning.</v>
+Prompt: Write a comparison plan for Chinese and Greek timekeeping evidence. Specify elapsed-time question, seconds, fixed vessel/hole/start level and three repeats. Explain how supplied shadow observations differ from your experiment and what neither can prove about ancient accuracy.
+Criteria: Same comparison questions for both cases; no direct China–Greece transmission claim; modern model is labeled.
+Response to difficulty: If timer is mistaken for navigation proof, identify its documented use and recheck; offer a protocol diagram without filling in reasoning.</v>
       </c>
       <c r="G11" s="11" t="str">
-        <v>Prepare adult-prepunched plastic vessels, trays, water, graduated measures/timers; no sharp student construction. Verify full CLOCK access and a Han source record before claiming source comparison ready.</v>
+        <v>Prepare adult-prepunched plastic vessels, trays, water, graduated measures/timers; no sharp student construction. Verify full CLOCK access and a Han source record before claiming source comparison ready. Carry saved private evidence and unresolved component notes to H3-W3-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H11" s="11" t="str">
-        <v>Teach / revisit: Han water clocks/sundials, Athenian court timer, astronomical patterns; elapsed-time versus time-of-day; historical evidence versus modern measurement.
-Practice: Select historical evidence from both societies; define elapsed-time question, fixed vessel/hole/start volume and repeated observations; predict limitations; read supplied shadow table.
+        <v>Teach / revisit: Plan a fair timekeeping comparison
+Practice: source/context reasoning through the project task.
 Check: Individual comparison plan naming sources, measurements/units, controls and evidence limits.
 Builds on: H3 context, source evaluation and measurement/graph entry check.</v>
       </c>
@@ -5474,10 +5500,10 @@
         <v>C3 Primary: D1.5.6-8, D3.2.6-8, D2.His.10.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="12" ht="186" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="12" ht="242" customHeight="1">
       <c r="A12" s="17" t="str">
         <v>H3-W3-G
 Week 3 | Group</v>
@@ -5487,27 +5513,28 @@
 Repeated elapsed-time observations; water-level/flow variability; comparison with supplied source-labeled shadow data.</v>
       </c>
       <c r="C12" s="15" t="str">
-        <v>The Met — Han Dynasty (206 BCE–220 CE); American School of Classical Studies at Athens — An Athenian Clepsydra
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+        <v>The Met — Han Dynasty (206 BCE–220 CE); University of St Andrews MacTutor — Timekeeping in the Ancient World: Water-clocks
+In class: 150–250 words of attributed teacher adaptation from Reread selected clock contexts; teacher-created shadow table and recorded class observations, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D12" s="13" t="str">
-        <v>Demonstrate timing a fixed drained volume and honest anomaly recording; changing water level can affect rate. Results describe this model.</v>
+        <v>Demonstrate timing a fixed drained volume and honest anomaly recording; changing water level can affect rate. Results describe this model. Example: For illustrative values 32,35,33 seconds, range=35−32=3 seconds. A changing water head may affect flow. One successful repeat still leaves construction and historical-use uncertainty.</v>
       </c>
       <c r="E12" s="13" t="str">
-        <v>Assemble teacher-prepared timer; record three short trials under consistent start conditions; compare variation and shadow-table constraints; draft one bounded historical/scientific comparison.</v>
+        <v>Teacher demonstrates/reset check; teams record three consistent-start trials, analyze range, compare supplied shadows, draft a bounded historical caption. Collect private interpretation; clean up. Full procedure in linked plan.</v>
       </c>
       <c r="F12" s="13" t="str">
         <v>Collect: Each student records/reads a trial, explains a data pattern and states one limit on historical inference.
-Judge: Units and repeat conditions explicit; scientific observations separated from historical claims; no civilization accuracy ranking from a classroom model.
-Feedback/support: If invented perfect repeats replace measurements, keep anomalies and recheck inference; accessible direct timing/recording participation or labeled supplied data.</v>
+Prompt: Report the three trial times with units and range. Explain one reason variation might occur and one shadow-table constraint. Use one source from each society to distinguish documented historical use from your modern model's result.
+Criteria: Units and repeat conditions explicit; scientific observations separated from historical claims; no civilization accuracy ranking from a classroom model.
+Response to difficulty: If invented perfect repeats replace measurements, keep anomalies and recheck inference; accessible direct timing/recording participation or labeled supplied data.</v>
       </c>
       <c r="G12" s="13" t="str">
-        <v>Budget setup/model 20, project trials/analysis 40, individual comparison 20, cleanup 10 minutes. Confirm kit access and trial durations before detailed production.</v>
+        <v>Budget setup/model 20, project trials/analysis 40, individual comparison 20, cleanup 10 minutes. Confirm kit access and trial durations before detailed production. Carry saved private evidence and unresolved component notes to H3-W4-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H12" s="13" t="str">
-        <v>Teach / revisit: Repeated elapsed-time observations; water-level/flow variability; comparison with supplied source-labeled shadow data.
-Practice: Assemble teacher-prepared timer; record three short trials under consistent start conditions; compare variation and shadow-table constraints; draft one bounded historical/scientific comparison.
+        <v>Teach / revisit: Test a modern timer and interpret its limits
+Practice: source/context reasoning through the project task.
 Check: Each student records/reads a trial, explains a data pattern and states one limit on historical inference.
 Builds on: W3-I plan; no assumed completion of science course.</v>
       </c>
@@ -5515,10 +5542,10 @@
         <v>C3 Primary: D3.3.6-8, D2.His.10.6-8, D4.2.6-8
 Supporting: D3.1.6-8
 NCSS themes: T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="13" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="13" ht="228" customHeight="1">
       <c r="A13" s="16" t="str">
         <v>H3-W4-I
 Week 4 | Individual</v>
@@ -5529,26 +5556,27 @@
       </c>
       <c r="C13" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; The Met — Han Dynasty (206 BCE–220 CE); Science Museum — Ancient Greek Computing
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 5.1 Ancient China: Silk Road; 6.3 The Hellenistic Era: diffusion, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D13" s="11" t="str">
-        <v>Model evidence for a documented route versus unsupported transmission from similar objects; separate Han and Hellenistic timelines.</v>
+        <v>Model evidence for a documented route versus unsupported transmission from similar objects; separate Han and Hellenistic timelines. Example: A route with intermediaries can carry goods or ideas without a single direct journey. Similar shapes are weaker transmission evidence than dated contact plus shared technical features.</v>
       </c>
       <c r="E13" s="11" t="str">
-        <v>Annotate two exchange maps; add routes, society-context panels and timer data to the same display; critique one transmission claim.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate two exchange maps; add routes, society-context panels and timer data to the same display; critique one transmission claim. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F13" s="11" t="str">
         <v>Collect: Private route explanation and evidence-based comparison of exchange, with one similarity that does not prove borrowing.
-Judge: Networks include intermediaries and dates; historical contexts remain distinct; display carries both society evidence and experiment limit.
-Feedback/support: If one direct route joins every inventor, examine route chronology and recheck; provide source/date keys.</v>
+Prompt: Annotate Silk Road and Hellenistic exchange with dates/intermediaries, including Buddhism's spread and Alexander's context. Explain one exchange mechanism and why similar inventions alone cannot prove direct China–Greece borrowing.
+Criteria: Networks include intermediaries and dates; historical contexts remain distinct; display carries both society evidence and experiment limit.
+Response to difficulty: If one direct route joins every inventor, examine route chronology and recheck; provide source/date keys.</v>
       </c>
       <c r="G13" s="11" t="str">
-        <v>Prepare a fresh invention/source card; keep final display compact—two panels, shared map/timeline and one data/comparison table.</v>
+        <v>Prepare a fresh invention/source card; keep final display compact—two panels, shared map/timeline and one data/comparison table. Carry saved private evidence and unresolved component notes to H3-W4-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H13" s="11" t="str">
-        <v>Teach / revisit: Silk Road goods/Buddhist diffusion; Macedonia/Alexander/Hellenistic diffusion; dated networks and distinct chronology.
-Practice: Annotate two exchange maps; add routes, society-context panels and timer data to the same display; critique one transmission claim.
+        <v>Teach / revisit: Trace exchange and finish the paired display
+Practice: source/context reasoning through the project task.
 Check: Private route explanation and evidence-based comparison of exchange, with one similarity that does not prove borrowing.
 Builds on: Dynasties, Greek wars/ideas, timer evidence.</v>
       </c>
@@ -5556,10 +5584,10 @@
         <v>C3 Primary: D2.His.1.6-8, D3.3.6-8, D4.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T3, T8, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="14" ht="200" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="14" ht="242" customHeight="1">
       <c r="A14" s="17" t="str">
         <v>H3-W4-G
 Week 4 | Group</v>
@@ -5569,27 +5597,28 @@
 Paired display review; institutions, history, experiment limits and fresh source reasoning.</v>
       </c>
       <c r="C14" s="15" t="str">
-        <v>OpenStax — World History Volume 1, to 1500; The Met — Han Dynasty (206 BCE–220 CE); American School of Classical Studies at Athens — An Athenian Clepsydra; Science Museum — Ancient Greek Computing
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+        <v>OpenStax — World History Volume 1, to 1500; The Met — Han Dynasty (206 BCE–220 CE); University of St Andrews MacTutor — Timekeeping in the Ancient World: Water-clocks; Science Museum — Ancient Greek Computing
+In class: 150–250 words of attributed teacher adaptation from Reuse H3 contexts; held-back dated printing record, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D14" s="13" t="str">
-        <v>Model explaining how a source and measured observation answer different questions; critique explanation order.</v>
+        <v>Model explaining how a source and measured observation answer different questions; critique explanation order. Example: A fresh record dated 868 CE qualifies a Han printing caption. Use chronology to revise the attribution, while recognizing a surviving print does not itself prove the first invention date.</v>
       </c>
       <c r="E14" s="13" t="str">
-        <v>Teams give short demonstration/walkthroughs; each student explains China and Greece achievement/context; respond to a fresh dated source and revise comparison.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Teams give short demonstration/walkthroughs; each student explains China and Greece achievement/context; respond to a fresh dated source and revise comparison. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F14" s="13" t="str">
         <v>Collect: Private both-society explanation, data interpretation, institutional influence and evidence limit; team display separate.
-Judge: Neither society omitted; scientific comparison and historical corroboration both visible; science standards not automatically credited.
-Feedback/support: If polished display masks history gaps, use separate map/institution/conflict mini-checks and source clinic; record unresolved component.</v>
+Prompt: Explain a Chinese and a Greek achievement with institutional context and a source limit. Interpret a fresh dated invention record and your timer data. Revise the comparison without treating classroom results as a ranking of civilizations.
+Criteria: Neither society omitted; scientific comparison and historical corroboration both visible; science standards not automatically credited.
+Response to difficulty: If polished display masks history gaps, use separate map/institution/conflict mini-checks and source clinic; record unresolved component.</v>
       </c>
       <c r="G14" s="13" t="str">
-        <v>Archive individual history and measurement evidence; retain chronology concern for TN appendix.</v>
+        <v>Archive individual history and measurement evidence; retain chronology concern for TN appendix. Carry saved private evidence and unresolved component notes to H4-W1-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H14" s="13" t="str">
-        <v>Teach / revisit: Paired display review; institutions, history, experiment limits and fresh source reasoning.
-Practice: Teams give short demonstration/walkthroughs; each student explains China and Greece achievement/context; respond to a fresh dated source and revise comparison.
+        <v>Teach / revisit: Demonstrate and defend ancient science comparisons
+Practice: source/context reasoning through the project task.
 Check: Private both-society explanation, data interpretation, institutional influence and evidence limit; team display separate.
 Builds on: All H3 context, source and investigation work.</v>
       </c>
@@ -5597,7 +5626,7 @@
         <v>C3 Primary: D4.1.6-8, D4.5.6-8, D2.His.16.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T5, T8, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
       </c>
     </row>
     <row r="15">
@@ -5654,7 +5683,7 @@
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
     </row>
-    <row r="19" ht="102" customHeight="1">
+    <row r="19" ht="116" customHeight="1">
       <c r="A19" s="11" t="str">
         <v>H3-W1-I</v>
       </c>
@@ -5666,7 +5695,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D19" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -5674,7 +5703,7 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" ht="102" customHeight="1">
+    <row r="20" ht="116" customHeight="1">
       <c r="A20" s="13" t="str">
         <v>H3-W1-G</v>
       </c>
@@ -5686,7 +5715,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D20" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -5694,7 +5723,7 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" ht="102" customHeight="1">
+    <row r="21" ht="116" customHeight="1">
       <c r="A21" s="11" t="str">
         <v>H3-W2-I</v>
       </c>
@@ -5706,7 +5735,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D21" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -5714,7 +5743,7 @@
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" ht="102" customHeight="1">
+    <row r="22" ht="116" customHeight="1">
       <c r="A22" s="13" t="str">
         <v>H3-W2-G</v>
       </c>
@@ -5726,7 +5755,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D22" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -5734,7 +5763,7 @@
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" ht="102" customHeight="1">
+    <row r="23" ht="116" customHeight="1">
       <c r="A23" s="11" t="str">
         <v>H3-W3-I</v>
       </c>
@@ -5746,7 +5775,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D23" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -5754,7 +5783,7 @@
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
     </row>
-    <row r="24" ht="102" customHeight="1">
+    <row r="24" ht="116" customHeight="1">
       <c r="A24" s="13" t="str">
         <v>H3-W3-G</v>
       </c>
@@ -5766,7 +5795,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D24" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -5774,7 +5803,7 @@
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
     </row>
-    <row r="25" ht="102" customHeight="1">
+    <row r="25" ht="116" customHeight="1">
       <c r="A25" s="11" t="str">
         <v>H3-W4-I</v>
       </c>
@@ -5786,7 +5815,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D25" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -5794,7 +5823,7 @@
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
     </row>
-    <row r="26" ht="102" customHeight="1">
+    <row r="26" ht="116" customHeight="1">
       <c r="A26" s="13" t="str">
         <v>H3-W4-G</v>
       </c>
@@ -5806,7 +5835,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D26" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -5870,7 +5899,7 @@
     </row>
     <row r="31" ht="116" customHeight="1">
       <c r="A31" s="11" t="str">
-        <v>Project outline</v>
+        <v>Detailed project plan</v>
       </c>
       <c r="B31" s="14" t="str">
         <v>H3 Ancient Science: Inventions, Sky and Navigation</v>
@@ -5879,7 +5908,7 @@
         <v>One paired China–Greece display with map/timeline, historical source panels, comparison table and investigation data; a short demonstration and individual explanation. Shadow data are supplied; the one practical investigation tests a water timer.</v>
       </c>
       <c r="D31" s="11" t="str">
-        <v>Step 4 outline exists; detailed Step 5 lessons pending.</v>
+        <v>Eight detailed Step 5 plans developed; Step 6 materials remain.</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -5898,7 +5927,7 @@
         <v>Teacher background: early humans, river-valley societies, ancient Israel/India/China/Greece/Rome. Select topic sections and primary-source boxes; prepare short attributed student adaptations.</v>
       </c>
       <c r="D32" s="13" t="str">
-        <v>Teacher reference located; exact excerpts, dates, image rights, reading fit and source packets remain Step 5/6 work. Do not assign whole college chapters.</v>
+        <v>Named section selections specified in all 32 detailed plans. Bounded Grade 6 adaptations and source boxes remain Step 6; do not assign whole college chapters.</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -5925,18 +5954,18 @@
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
     </row>
-    <row r="34" ht="74" customHeight="1">
+    <row r="34" ht="102" customHeight="1">
       <c r="A34" s="13" t="str">
         <v>CLOCK</v>
       </c>
       <c r="B34" s="15" t="str">
-        <v>American School of Classical Studies at Athens — An Athenian Clepsydra</v>
+        <v>University of St Andrews MacTutor — Timekeeping in the Ancient World: Water-clocks</v>
       </c>
       <c r="C34" s="13" t="str">
-        <v>Archaeological scholarly account of Athenian court timing; isolate one object image/description and its reconstruction limits.</v>
+        <v>Daniel Mintz, April 2007. Opening through Athenian judicial use; flow/pressure explanation. Pair with Met Han timekeeping interpretation. Modern scholarly account, not an ancient eyewitness.</v>
       </c>
       <c r="D34" s="13" t="str">
-        <v>Search-indexed research source; full PDF retrieval failed. Access and precise page selection conditional before Step 5.</v>
+        <v>Teacher text reviewed; accessible student adaptation remains Step 6. Archaeological primary object selection remains conditional.</v>
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -6787,11 +6816,11 @@
     </row>
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="3" t="str">
-        <v>Step 4 block outlines</v>
+        <v>Step 5 teacher plans</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="str">
-        <v>Detailed procedures, exact source excerpts, examples and assessment prompts remain Step 5 work.</v>
+        <v>Full procedures, worked examples, private prompts and clocks in linked plans; Step 6 packets and trials remain.</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -6840,7 +6869,7 @@
         <v>Standards - national</v>
       </c>
     </row>
-    <row r="7" ht="172" customHeight="1">
+    <row r="7" ht="214" customHeight="1">
       <c r="A7" s="16" t="str">
         <v>H4-W1-I
 Week 1 | Individual</v>
@@ -6851,26 +6880,27 @@
       </c>
       <c r="C7" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 6.4 The Roman Republic: institutions, law, social groups and geography, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D7" s="11" t="str">
-        <v>Model offices/participation without calling Rome a modern inclusive democracy; place later Constantinople on a dated map layer.</v>
+        <v>Model offices/participation without calling Rome a modern inclusive democracy; place later Constantinople on a dated map layer. Example: An institutional diagram shows a check on officials but also eligibility limits. A road/marine route may help movement; access alone does not explain every conquest.</v>
       </c>
       <c r="E7" s="11" t="str">
-        <v>Annotate geographic growth map; diagram institutions and eligible participation; compare a rule to affected social groups.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate geographic growth map; diagram institutions and eligible participation; compare a rule to affected social groups. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F7" s="11" t="str">
         <v>Collect: Individual map plus institution/participation explanation including excluded groups.
-Judge: Dates/layers explicit; government functions and social limits clear; geography connected to growth.
-Feedback/support: If checks imply equality for everyone, use participation matrix and recheck; accessible map/source chunks.</v>
+Prompt: Label Rome's six features, dating Constantinople as a later capital. Diagram republic branches/checks and Twelve Tables; explain patrician/plebeian/enslaved participation and a geographic mechanism of expansion.
+Criteria: Dates/layers explicit; government functions and social limits clear; geography connected to growth.
+Response to difficulty: If checks imply equality for everyone, use participation matrix and recheck; accessible map/source chunks.</v>
       </c>
       <c r="G7" s="11" t="str">
-        <v>Prepare verified Twelve Tables translation and dated maps; reuse H3 citizenship comparison.</v>
+        <v>Prepare verified Twelve Tables translation and dated maps; reuse H3 citizenship comparison. Carry saved private evidence and unresolved component notes to H4-W1-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H7" s="11" t="str">
-        <v>Teach / revisit: Tiber, Rome, Italy/Alps, Mediterranean, Constantinople later timeline; geography/growth; patricians, plebeians and enslaved people; republican offices, Senate/assemblies, checks, participation and Twelve Tables.
-Practice: Annotate geographic growth map; diagram institutions and eligible participation; compare a rule to affected social groups.
+        <v>Teach / revisit: Locate Rome and explain the republic
+Practice: source/context reasoning through the project task.
 Check: Individual map plus institution/participation explanation including excluded groups.
 Builds on: Greek polis and source-based comparison.</v>
       </c>
@@ -6878,10 +6908,10 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.Civ.6.6-8, D2.His.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T3, T4, T5, T6, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="8" ht="158" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="8" ht="214" customHeight="1">
       <c r="A8" s="17" t="str">
         <v>H4-W1-G
 Week 1 | Group</v>
@@ -6892,26 +6922,27 @@
       </c>
       <c r="C8" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 6.4 The Roman Republic: late republic; 6.5 The Age of Augustus: transition and Pax Romana, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D8" s="13" t="str">
-        <v>Compare a ruler image/claim to another account; trace structural tensions alongside leaders and trigger events.</v>
+        <v>Compare a ruler image/claim to another account; trace structural tensions alongside leaders and trigger events. Example: A ruler's public achievement account emphasizes success; compare a separate account before explaining transition. Caesar's dictatorship and Augustus's principate belong at different timeline points.</v>
       </c>
       <c r="E8" s="13" t="str">
-        <v>Build transition timeline; compare institutional change and source perspectives; add cause/effect evidence to council dossier.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Build transition timeline; compare institutional change and source perspectives; add cause/effect evidence to council dossier. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F8" s="13" t="str">
         <v>Collect: Private multi-factor transition explanation and ruler-source purpose inference.
-Judge: Distinguishes Caesar from Augustus and continuity from change; propaganda not treated as complete social evidence.
-Feedback/support: If one leader explains everything, add a structural evidence card and recheck; use dated actors/events.</v>
+Prompt: Sequence Caesar's military/popular power, dictatorship/assassination and Augustus/Pax Romana. Explain two interacting causes of institutional change and one continuity. Infer a ruler claim's audience/purpose using a contrasting account.
+Criteria: Distinguishes Caesar from Augustus and continuity from change; propaganda not treated as complete social evidence.
+Response to difficulty: If one leader explains everything, add a structural evidence card and recheck; use dated actors/events.</v>
       </c>
       <c r="G8" s="13" t="str">
-        <v>Select contrasting accounts and dated coin/inscription; preserve institutional chart for W4 synthesis.</v>
+        <v>Select contrasting accounts and dated coin/inscription; preserve institutional chart for W4 synthesis. Carry saved private evidence and unresolved component notes to H4-W2-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H8" s="13" t="str">
-        <v>Teach / revisit: Julius Caesar military leadership, popular support, dictatorship/assassination; Augustus and Pax Romana expansion and institutions.
-Practice: Build transition timeline; compare institutional change and source perspectives; add cause/effect evidence to council dossier.
+        <v>Teach / revisit: Explain republic-to-empire change
+Practice: source/context reasoning through the project task.
 Check: Private multi-factor transition explanation and ruler-source purpose inference.
 Builds on: Republic roles and evidence limitation.</v>
       </c>
@@ -6919,10 +6950,10 @@
         <v>C3 Primary: D2.His.1.6-8, D2.His.14.6-8, D2.His.6.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T5, T6 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="9" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="9" ht="228" customHeight="1">
       <c r="A9" s="16" t="str">
         <v>H4-W2-I
 Week 2 | Individual</v>
@@ -6933,26 +6964,27 @@
       </c>
       <c r="C9" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 7.1 The Daily Life of a Roman Family and 7.3 The Roman Economy: selected infrastructure/daily-life passages, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D9" s="11" t="str">
-        <v>Model infrastructure benefits and unequal access/costs; monument evidence cannot describe everyone’s daily life.</v>
+        <v>Model infrastructure benefits and unequal access/costs; monument evidence cannot describe everyone’s daily life. Example: An aqueduct moves water using a gradient; distribution depends on maintenance and decisions. A monumental arch shows construction technique without establishing equal household access.</v>
       </c>
       <c r="E9" s="11" t="str">
-        <v>Trace two infrastructure systems on a city diagram; explain remaining examples through a short annotated gallery; connect civic/religious use to daily experience.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Trace two infrastructure systems on a city diagram; explain remaining examples through a short annotated gallery; connect civic/religious use to daily experience. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F9" s="11" t="str">
         <v>Collect: Individual system explanation and attributed polytheism/context note.
-Judge: Explains function and human/environment effects; all named infrastructure appears; social differences recognized.
-Feedback/support: If drawings replace reasoning, add flow/use labels and recheck another structure; offer large diagrams.</v>
+Prompt: Explain two infrastructure systems using flow/use labels; identify functions of arches, aqueducts, bridges, domes, roads, sanitation and Colosseum. Connect polytheistic civic use and explain unequal benefits or costs.
+Criteria: Explains function and human/environment effects; all named infrastructure appears; social differences recognized.
+Response to difficulty: If drawings replace reasoning, add flow/use labels and recheck another structure; offer large diagrams.</v>
       </c>
       <c r="G9" s="11" t="str">
-        <v>No extra engineering build; select verified diagram/object sources and maintain the same dossier.</v>
+        <v>No extra engineering build; select verified diagram/object sources and maintain the same dossier. Carry saved private evidence and unresolved component notes to H4-W2-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H9" s="11" t="str">
-        <v>Teach / revisit: Arches, aqueducts, bridges, domes, roads, sanitation and Colosseum; work, distribution, trade and polytheistic practice.
-Practice: Trace two infrastructure systems on a city diagram; explain remaining examples through a short annotated gallery; connect civic/religious use to daily experience.
+        <v>Teach / revisit: Explain engineering and everyday life
+Practice: source/context reasoning through the project task.
 Check: Individual system explanation and attributed polytheism/context note.
 Builds on: H1 technology and H3 model/historical evidence distinction.</v>
       </c>
@@ -6960,10 +6992,10 @@
         <v>C3 Primary: D2.Geo.4.6-8, D2.Civ.6.6-8, D4.2.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T3, T7, T8 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="10" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="10" ht="228" customHeight="1">
       <c r="A10" s="17" t="str">
         <v>H4-W2-G
 Week 2 | Group</v>
@@ -6974,26 +7006,27 @@
       </c>
       <c r="C10" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 7.4 Religion in the Roman Empire: religious beliefs, Christianity and Jewish communities, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D10" s="13" t="str">
-        <v>Use the common religion template from H2; distinguish faith claims from historical analysis and explain multiple diaspora phases.</v>
+        <v>Use the common religion template from H2; distinguish faith claims from historical analysis and explain multiple diaspora phases. Example: A sacred account expresses a faith claim; historical spread uses dated movement and institution evidence. A diaspora map should distinguish separate conflicts and continuing communities.</v>
       </c>
       <c r="E10" s="13" t="str">
-        <v>Annotate religion/context cards; map dated displacement/spread; compare two attributed accounts without devotional performance.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Annotate religion/context cards; map dated displacement/spread; compare two attributed accounts without devotional performance. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F10" s="13" t="str">
         <v>Collect: Private Christianity profile and source-based diaspora cause/movement explanation.
-Judge: Beliefs are accurately attributed; political conflict and movement dates are not collapsed into one expulsion or all-Jewish departure.
-Feedback/support: If sacred account becomes automatic modern historical proof, classify source purpose and corroborate; glossary and neutral response options.</v>
+Prompt: Complete a Christianity profile naming Jesus, Paul, Bible, monotheism, forgiveness, eternal life and Messiah as attributed beliefs. Explain a dated Jewish diaspora phase using political conflict and movement evidence; avoid one universal departure narrative.
+Criteria: Beliefs are accurately attributed; political conflict and movement dates are not collapsed into one expulsion or all-Jewish departure.
+Response to difficulty: If sacred account becomes automatic modern historical proof, classify source purpose and corroborate; glossary and neutral response options.</v>
       </c>
       <c r="G10" s="13" t="str">
-        <v>Prepare sensitive, scholarly source selection and timeline; no present-day group blame.</v>
+        <v>Prepare sensitive, scholarly source selection and timeline; no present-day group blame. Carry saved private evidence and unresolved component notes to H4-W3-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H10" s="13" t="str">
-        <v>Teach / revisit: Christianity: Jesus/Paul, Bible, monotheism, sin/forgiveness, eternal life, Messiah; historical spread/persecution and imperial change; Roman/Jewish conflicts and dispersal.
-Practice: Annotate religion/context cards; map dated displacement/spread; compare two attributed accounts without devotional performance.
+        <v>Teach / revisit: Contextualize Christianity and Jewish diaspora
+Practice: source/context reasoning through the project task.
 Check: Private Christianity profile and source-based diaspora cause/movement explanation.
 Builds on: H2 Judaism and respectful religious-source inquiry.</v>
       </c>
@@ -7001,10 +7034,10 @@
         <v>C3 Primary: D2.His.4.6-8, D2.His.6.6-8, D3.2.6-8
 Supporting: D3.1.6-8
 NCSS themes: T1, T4, T5, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="11" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="11" ht="214" customHeight="1">
       <c r="A11" s="16" t="str">
         <v>H4-W3-I
 Week 3 | Individual</v>
@@ -7015,26 +7048,27 @@
       </c>
       <c r="C11" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 10.1 The Eastward Shift: Constantine, regional division and eastern continuation, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D11" s="11" t="str">
-        <v>Model changing dated boundaries and multiple stages of division; 476 in the West does not end every Roman institution.</v>
+        <v>Model changing dated boundaries and multiple stages of division; 476 in the West does not end every Roman institution. Example: A dated eastern capital map preserves Roman administration after western political collapse. Changing boundaries and ongoing institutions can occur together.</v>
       </c>
       <c r="E11" s="11" t="str">
-        <v>Layer empire maps; identify capital-location factors; sort continuity/change evidence for eastern/western regions.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Layer empire maps; identify capital-location factors; sort continuity/change evidence for eastern/western regions. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F11" s="11" t="str">
         <v>Collect: Individual division map and explanation of one continuity and two capital/governance factors.
-Judge: Distinguishes division from western collapse; East continues; time/place shapes cause.
-Feedback/support: If a single map becomes timeless, add dates and recheck layers; use paired maps with consistent scale.</v>
+Prompt: Compare dated East/West maps, division and Constantine's capital. Explain two governance/location factors, one eastern continuity and why western collapse does not mean all Roman institutions ended.
+Criteria: Distinguishes division from western collapse; East continues; time/place shapes cause.
+Response to difficulty: If a single map becomes timeless, add dates and recheck layers; use paired maps with consistent scale.</v>
       </c>
       <c r="G11" s="11" t="str">
-        <v>Prepare map dates and source captions; save pressures for cause-ranking session.</v>
+        <v>Prepare map dates and source captions; save pressures for cause-ranking session. Carry saved private evidence and unresolved component notes to H4-W3-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H11" s="11" t="str">
-        <v>Teach / revisit: Constantine/Constantinople; administrative division versus relocation; East/West and Byzantine continuation; territory/governing pressures.
-Practice: Layer empire maps; identify capital-location factors; sort continuity/change evidence for eastern/western regions.
+        <v>Teach / revisit: Map division and eastern continuation
+Practice: source/context reasoning through the project task.
 Check: Individual division map and explanation of one continuity and two capital/governance factors.
 Builds on: Rome institutions, geography and regional comparison.</v>
       </c>
@@ -7042,10 +7076,10 @@
         <v>C3 Primary: D2.Geo.1.6-8, D2.His.2.6-8, D2.His.14.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T3, T5, T6 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="12" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="12" ht="228" customHeight="1">
       <c r="A12" s="17" t="str">
         <v>H4-W3-G
 Week 3 | Group</v>
@@ -7056,26 +7090,27 @@
       </c>
       <c r="C12" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from 10.1 The Eastward Shift: pressures and western collapse; contrast interpretations within the account, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D12" s="13" t="str">
-        <v>Model comparing the explanatory reach of causes; avoid a single invasion-only or moral-decline explanation.</v>
+        <v>Model comparing the explanatory reach of causes; avoid a single invasion-only or moral-decline explanation. Example: Military pressure and revenue loss may reinforce one another. Ranking a cause requires explaining its reach and interaction, rather than declaring it more interesting.</v>
       </c>
       <c r="E12" s="13" t="str">
-        <v>Compare three bounded interpretations with evidence; make a causal web; weigh two causes and challenge unsupported claims.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Compare three bounded interpretations with evidence; make a causal web; weigh two causes and challenge unsupported claims. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F12" s="13" t="str">
         <v>Collect: Private cause-ranking argument with evidence, a competing view and limitation.
-Judge: Multiple interacting causes; relative influence justified; distinguishes evidence from a rhetorical moral claim.
-Feedback/support: If ranking is personal preference, require a sourced mechanism then recheck a new cause; provide an evidence/cause chart.</v>
+Prompt: Rank two influences on western collapse using evidence and mechanisms; incorporate a third interacting cause, a competing explanation and a source limit. Explain why invasion alone or unsupported moral decline is insufficient.
+Criteria: Multiple interacting causes; relative influence justified; distinguishes evidence from a rhetorical moral claim.
+Response to difficulty: If ranking is personal preference, require a sourced mechanism then recheck a new cause; provide an evidence/cause chart.</v>
       </c>
       <c r="G12" s="13" t="str">
-        <v>Select contrasting historian arguments and provenance; reserve revision for W4-I.</v>
+        <v>Select contrasting historian arguments and provenance; reserve revision for W4-I. Carry saved private evidence and unresolved component notes to H4-W4-I; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H12" s="13" t="str">
-        <v>Teach / revisit: Large territory, political instability/corruption, economic pressures, Germanic groups and military conflict; relative cause influence and evidence limits.
-Practice: Compare three bounded interpretations with evidence; make a causal web; weigh two causes and challenge unsupported claims.
+        <v>Teach / revisit: Weigh explanations for western collapse
+Practice: source/context reasoning through the project task.
 Check: Private cause-ranking argument with evidence, a competing view and limitation.
 Builds on: Division/continuation and source credibility.</v>
       </c>
@@ -7083,10 +7118,10 @@
         <v>C3 Primary: D2.His.15.6-8, D3.3.6-8, D4.4.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T6, T7, T9 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="13" ht="172" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="13" ht="214" customHeight="1">
       <c r="A13" s="16" t="str">
         <v>H4-W4-I
 Week 4 | Individual</v>
@@ -7097,26 +7132,27 @@
       </c>
       <c r="C13" s="14" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from Reuse H4 dossier and dated maps, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D13" s="11" t="str">
-        <v>Model an evidence council discussing actual historical causes; conjectured policy outcomes, if mentioned, are labeled counterfactual.</v>
+        <v>Model an evidence council discussing actual historical causes; conjectured policy outcomes, if mentioned, are labeled counterfactual. Example: An account that says invasions caused everything omits institutional and economic mechanisms. Add a sourced interaction and eastern contrast instead of a longer list of unsupported causes.</v>
       </c>
       <c r="E13" s="11" t="str">
-        <v>Finish existing dossier; individually write a bounded multi-cause account; critique source credibility and sequence; revise one argument.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Finish existing dossier; individually write a bounded multi-cause account; critique source credibility and sequence; revise one argument. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F13" s="11" t="str">
         <v>Collect: Independent 200–300-word or equivalent causal account with multiple sources, limitation and revision.
-Judge: Historical outcomes accurate; East/West distinction preserved; evidence addresses causes and institutional change.
-Feedback/support: If team consensus replaces private learning, collect independent account first; scaffold organization without supplying the claim.</v>
+Prompt: Write an independent 200–300-word or equivalent account linking republic-to-empire change and western collapse. Use multiple sources, distinguish eastern continuation and address a competing explanation; revise reasoning after source/sequence critique.
+Criteria: Historical outcomes accurate; East/West distinction preserved; evidence addresses causes and institutional change.
+Response to difficulty: If team consensus replaces private learning, collect independent account first; scaffold organization without supplying the claim.</v>
       </c>
       <c r="G13" s="11" t="str">
-        <v>Prepare a fresh map/account check and a contribution roster; no game or alternative-history victory scoring.</v>
+        <v>Prepare a fresh map/account check and a contribution roster; no game or alternative-history victory scoring. Carry saved private evidence and unresolved component notes to H4-W4-G; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H13" s="11" t="str">
-        <v>Teach / revisit: Synthesize republic, empire, infrastructure, religion, diaspora, division and fall; evaluate arguments and coherent explanations.
-Practice: Finish existing dossier; individually write a bounded multi-cause account; critique source credibility and sequence; revise one argument.
+        <v>Teach / revisit: Prepare the evidence council
+Practice: source/context reasoning through the project task.
 Check: Independent 200–300-word or equivalent causal account with multiple sources, limitation and revision.
 Builds on: All H4 institutional, geographic and causal work.</v>
       </c>
@@ -7124,10 +7160,10 @@
         <v>C3 Primary: D2.His.16.6-8, D4.1.6-8, D4.5.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T5, T6, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
-      </c>
-    </row>
-    <row r="14" ht="186" customHeight="1">
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
+      </c>
+    </row>
+    <row r="14" ht="214" customHeight="1">
       <c r="A14" s="17" t="str">
         <v>H4-W4-G
 Week 4 | Group</v>
@@ -7138,26 +7174,27 @@
       </c>
       <c r="C14" s="15" t="str">
         <v>OpenStax — World History Volume 1, to 1500; British Museum — Greece and Rome
-Planning limit: 150–250 words of new adapted prose plus up to two images/maps/source cards. Exact excerpts, provenance and access pending; essential reading stays in class.
-Open for the linked outline and source details.</v>
+In class: 150–250 words of attributed teacher adaptation from Held-back account/map; reuse H4 dossier, with at most two map/image/source cards. Read once for context and reread the cited clue; preview 3–5 topic terms. Adaptations are proposed materials, not finished packets.
+Open the linked full plan for procedures, assessment and source details.</v>
       </c>
       <c r="D14" s="13" t="str">
-        <v>Model civil critique: identify claim, relevant source, limitation and evidence that would change the conclusion.</v>
+        <v>Model civil critique: identify claim, relevant source, limitation and evidence that would change the conclusion. Example: A fresh account can strengthen one causal mechanism while leaving another uncertain. Civil critique asks what evidence would change a claim and avoids attacking its author personally.</v>
       </c>
       <c r="E14" s="13" t="str">
-        <v>Teams present actual-history explanations; every student responds to a question; independently analyze a fresh source and revise the causal account.</v>
+        <v>1. Read/mark evidence. 2. Guided source turn. 3. Teams present actual-history explanations; every student responds to a question; independently analyze a fresh source and revise the causal account. 4. Private check. 5. Revise and save. Full procedures and clock in linked plan.</v>
       </c>
       <c r="F14" s="13" t="str">
         <v>Collect: Teacher-recorded response, fresh source inference and independent revision; team council quality assessed separately.
-Judge: Civil discussion and supported reasoning; new evidence changes or sustains a conclusion for a stated reason.
-Feedback/support: If performance masks missing history, use targeted map/chronology/source recheck; record remaining learning for the next course.</v>
+Prompt: Respond privately to a held-back historical account/map: identify claim, context, credibility and a limit. Explain whether it changes your causal account. Support one council response with evidence and record your own revision.
+Criteria: Civil discussion and supported reasoning; new evidence changes or sustains a conclusion for a stated reason.
+Response to difficulty: If performance masks missing history, use targeted map/chronology/source recheck; record remaining learning for the next course.</v>
       </c>
       <c r="G14" s="13" t="str">
-        <v>Archive inquiry growth and unresolved content; use a class-approved exhibit correction as a bounded civic practice, without a full informed-action indicator claim.</v>
+        <v>Archive inquiry growth and unresolved content; use a class-approved exhibit correction as a bounded civic practice, without a full informed-action indicator claim. Carry saved private evidence and unresolved component notes to the next history course; use its opening retrieval/clinic budget for a fresh check. Final unresolved needs go in the receiving teacher record. No homework required.</v>
       </c>
       <c r="H14" s="13" t="str">
-        <v>Teach / revisit: Evidence council, fresh historical source interpretation and course-wide inquiry reflection.
-Practice: Teams present actual-history explanations; every student responds to a question; independently analyze a fresh source and revise the causal account.
+        <v>Teach / revisit: Hold the council and apply new evidence
+Practice: source/context reasoning through the project task.
 Check: Teacher-recorded response, fresh source inference and independent revision; team council quality assessed separately.
 Builds on: All-course source selection, comparison and causation.</v>
       </c>
@@ -7165,7 +7202,7 @@
         <v>C3 Primary: D4.1.6-8, D4.4.6-8, D2.His.10.6-8
 Supporting: D3.1.6-8
 NCSS themes: T2, T9, T10 (local labels).
-Confirmed at outline level; exact source-dependent interpretations conditional. Whole-band coverage and detailed plans are not claimed.</v>
+Step 5 teaching/practice/private check specified. Source-dependent claims Conditional until packets verified; selected contributions only.</v>
       </c>
     </row>
     <row r="15">
@@ -7222,7 +7259,7 @@
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
     </row>
-    <row r="19" ht="102" customHeight="1">
+    <row r="19" ht="116" customHeight="1">
       <c r="A19" s="11" t="str">
         <v>H4-W1-I</v>
       </c>
@@ -7234,7 +7271,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D19" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -7242,7 +7279,7 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" ht="102" customHeight="1">
+    <row r="20" ht="116" customHeight="1">
       <c r="A20" s="13" t="str">
         <v>H4-W1-G</v>
       </c>
@@ -7254,7 +7291,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D20" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -7262,7 +7299,7 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" ht="102" customHeight="1">
+    <row r="21" ht="116" customHeight="1">
       <c r="A21" s="11" t="str">
         <v>H4-W2-I</v>
       </c>
@@ -7274,7 +7311,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D21" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -7282,7 +7319,7 @@
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" ht="102" customHeight="1">
+    <row r="22" ht="116" customHeight="1">
       <c r="A22" s="13" t="str">
         <v>H4-W2-G</v>
       </c>
@@ -7294,7 +7331,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D22" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -7302,7 +7339,7 @@
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" ht="102" customHeight="1">
+    <row r="23" ht="116" customHeight="1">
       <c r="A23" s="11" t="str">
         <v>H4-W3-I</v>
       </c>
@@ -7314,7 +7351,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D23" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -7322,7 +7359,7 @@
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
     </row>
-    <row r="24" ht="102" customHeight="1">
+    <row r="24" ht="116" customHeight="1">
       <c r="A24" s="13" t="str">
         <v>H4-W3-G</v>
       </c>
@@ -7334,7 +7371,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D24" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -7342,7 +7379,7 @@
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
     </row>
-    <row r="25" ht="102" customHeight="1">
+    <row r="25" ht="116" customHeight="1">
       <c r="A25" s="11" t="str">
         <v>H4-W4-I</v>
       </c>
@@ -7354,7 +7391,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D25" s="11" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -7362,7 +7399,7 @@
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
     </row>
-    <row r="26" ht="102" customHeight="1">
+    <row r="26" ht="116" customHeight="1">
       <c r="A26" s="13" t="str">
         <v>H4-W4-G</v>
       </c>
@@ -7374,7 +7411,7 @@
         <v>D3.1.6-8</v>
       </c>
       <c r="D26" s="13" t="str">
-        <v>Confirmed in the Step 4 outline for the specified contribution; source-dependent interpretations conditional until exact selections are verified. Detailed procedures and fresh assessment prompts remain Step 5.</v>
+        <v>Specified in Step 5: explicit model/review, project practice and the private prompt above support the listed selected contributions. Materials and observed attainment remain unverified. Topic-dependent source claims are conditional until the attributed packet is checked.</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -7438,7 +7475,7 @@
     </row>
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="11" t="str">
-        <v>Project outline</v>
+        <v>Detailed project plan</v>
       </c>
       <c r="B31" s="14" t="str">
         <v>H4 Rome: Republic to Division</v>
@@ -7447,7 +7484,7 @@
         <v>One team council dossier with map/timeline, institutional comparison and causal evidence chart. Each student submits a short independent multi-cause account and fresh-source revision.</v>
       </c>
       <c r="D31" s="11" t="str">
-        <v>Step 4 outline exists; detailed Step 5 lessons pending.</v>
+        <v>Eight detailed Step 5 plans developed; Step 6 materials remain.</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -7466,7 +7503,7 @@
         <v>Teacher background: early humans, river-valley societies, ancient Israel/India/China/Greece/Rome. Select topic sections and primary-source boxes; prepare short attributed student adaptations.</v>
       </c>
       <c r="D32" s="13" t="str">
-        <v>Teacher reference located; exact excerpts, dates, image rights, reading fit and source packets remain Step 5/6 work. Do not assign whole college chapters.</v>
+        <v>Named section selections specified in all 32 detailed plans. Bounded Grade 6 adaptations and source boxes remain Step 6; do not assign whole college chapters.</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>

</xml_diff>